<commit_message>
Record Marrakech nights at EUR 80 each and Budapest hostel booking
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FbPxpFjYDQnzNa7KTrLMWP
</commit_message>
<xml_diff>
--- a/Eurasia/Roteiro_Eurasia.xlsx
+++ b/Eurasia/Roteiro_Eurasia.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="546" uniqueCount="362">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="549" uniqueCount="365">
   <si>
     <t xml:space="preserve">Itinerário de Voos</t>
   </si>
@@ -466,33 +466,42 @@
     <t xml:space="preserve">Sai ~13:30 (22/10)</t>
   </si>
   <si>
+    <t xml:space="preserve">Segunda noite no mesmo riad. Pagamento em dinheiro (MAD).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Budapeste</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chega 20:30 (22/10) / sai ~09:45 (25/10)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Distrito VI (Terézváros)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Wombat's City Hostel</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Trip.com 20261022212925274204002979</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pago</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Wombat's City Hostel, Király u. 20, 1061 Budapeste. 1 cama, 3 noites. Check-in a partir das 14:00; check-out até 10:00. Valor: pagamento Trip.com de 22/10 (confirmar se é desta reserva).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Baku</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chega ~16:30 (25/10) / sai ~18:00 (28/10)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cidade Velha (Icherisheher) ou Nizami</t>
+  </si>
+  <si>
     <t xml:space="preserve">Pendente</t>
   </si>
   <si>
-    <t xml:space="preserve">URGENTE: a reserva atual cobre só 1 noite. Tentar estender no mesmo riad (21 a 22/10).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Budapeste</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Chega 20:30 (22/10) / sai ~09:45 (25/10)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Distrito VII (bairro judeu) ou V</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Região dos ruin bars; boa ligação de metrô.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Baku</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Chega ~16:30 (25/10) / sai ~18:00 (28/10)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cidade Velha (Icherisheher) ou Nizami</t>
-  </si>
-  <si>
     <t xml:space="preserve">Pedir para guardar as mochilas no dia 28 até a saída para o aeroporto.</t>
   </si>
   <si>
@@ -667,7 +676,7 @@
     <t xml:space="preserve">Praça Jemaa el-Fna ao pôr do sol; jantar num terraço.</t>
   </si>
   <si>
-    <t xml:space="preserve">Majorelle exige ingresso online com horário. Pernoite 21/10 ainda sem reserva.</t>
+    <t xml:space="preserve">Majorelle exige ingresso online com horário.</t>
   </si>
   <si>
     <t xml:space="preserve">qui</t>
@@ -946,10 +955,7 @@
     <t xml:space="preserve">Reservar 2ª noite Marraquexe (21 a 22/10)</t>
   </si>
   <si>
-    <t xml:space="preserve">HOJE</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Reserva atual cobre só 1 noite. Tentar estender no mesmo riad.</t>
+    <t xml:space="preserve">Mesmo riad, € 80.</t>
   </si>
   <si>
     <t xml:space="preserve">Sacar dirham (MAD) para pagar o riad</t>
@@ -958,61 +964,64 @@
     <t xml:space="preserve">Na chegada</t>
   </si>
   <si>
-    <t xml:space="preserve">€ 84,97 pagos em dinheiro na moeda local; sacar no caixa eletrônico do aeroporto de Marraquexe.</t>
+    <t xml:space="preserve">€ 80 por noite (€ 160 no total) pagos em dinheiro na moeda local.</t>
   </si>
   <si>
     <t xml:space="preserve">Reservar hostel Budapeste (22 a 25/10)</t>
   </si>
   <si>
+    <t xml:space="preserve">Wombat's City Hostel (1 cama). Confirmar se os meninos têm reserva própria.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Reservar hostel Baku (25 a 28/10)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Até 23/10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ver aba Hospedagem.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Reservar hostel Tbilisi (grupo 28 a 31/10 + Diego 31/10 a 01/11)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Até 25/10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Check-in ~22:30 no dia 28. Ver aba Hospedagem.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Reservar hostel Atenas (31/10 a 03/11)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Até 28/10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Média</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Reservar pernoite São Paulo (04 a 05/11)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Até 01/11</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Se não houver onde ficar. Ver aba Hospedagem.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ingresso Jardim Majorelle (21/10)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hoje</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Só online, com horário marcado.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Visita guiada Parlamento de Budapeste (23/10)</t>
+  </si>
+  <si>
     <t xml:space="preserve">21/10</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ver aba Hospedagem.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Reservar hostel Baku (25 a 28/10)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Até 23/10</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Reservar hostel Tbilisi (grupo 28 a 31/10 + Diego 31/10 a 01/11)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Até 25/10</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Check-in ~22:30 no dia 28. Ver aba Hospedagem.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Reservar hostel Atenas (31/10 a 03/11)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Até 28/10</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Média</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Reservar pernoite São Paulo (04 a 05/11)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Até 01/11</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Se não houver onde ficar. Ver aba Hospedagem.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ingresso Jardim Majorelle (21/10)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Hoje</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Só online, com horário marcado.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Visita guiada Parlamento de Budapeste (23/10)</t>
   </si>
   <si>
     <t xml:space="preserve">Esgota com antecedência; escolher horário em inglês ou espanhol.</t>
@@ -2409,7 +2418,7 @@
         <v>143</v>
       </c>
       <c r="I5" s="12" t="n">
-        <v>84.97</v>
+        <v>80</v>
       </c>
       <c r="J5" s="4" t="s">
         <v>144</v>
@@ -2418,7 +2427,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="10" t="s">
         <v>139</v>
       </c>
@@ -2438,19 +2447,23 @@
       <c r="F6" s="5" t="s">
         <v>141</v>
       </c>
-      <c r="G6" s="6"/>
+      <c r="G6" s="6" t="s">
+        <v>142</v>
+      </c>
       <c r="H6" s="6"/>
-      <c r="I6" s="14"/>
+      <c r="I6" s="12" t="n">
+        <v>80</v>
+      </c>
       <c r="J6" s="4" t="s">
+        <v>144</v>
+      </c>
+      <c r="K6" s="5" t="s">
         <v>147</v>
       </c>
-      <c r="K6" s="13" t="s">
+    </row>
+    <row r="7" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="10" t="s">
         <v>148</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="10" t="s">
-        <v>149</v>
       </c>
       <c r="B7" s="11" t="n">
         <v>46317</v>
@@ -2463,24 +2476,30 @@
         <v>3</v>
       </c>
       <c r="E7" s="5" t="s">
+        <v>149</v>
+      </c>
+      <c r="F7" s="5" t="s">
         <v>150</v>
       </c>
-      <c r="F7" s="5" t="s">
+      <c r="G7" s="6" t="s">
         <v>151</v>
       </c>
-      <c r="G7" s="6"/>
-      <c r="H7" s="6"/>
-      <c r="I7" s="14"/>
+      <c r="H7" s="6" t="s">
+        <v>152</v>
+      </c>
+      <c r="I7" s="14" t="n">
+        <v>840.92</v>
+      </c>
       <c r="J7" s="4" t="s">
-        <v>147</v>
+        <v>153</v>
       </c>
       <c r="K7" s="5" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="10" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="B8" s="11" t="n">
         <v>46320</v>
@@ -2493,24 +2512,24 @@
         <v>3</v>
       </c>
       <c r="E8" s="5" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="F8" s="5" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="G8" s="6"/>
       <c r="H8" s="6"/>
       <c r="I8" s="14"/>
       <c r="J8" s="4" t="s">
-        <v>147</v>
+        <v>158</v>
       </c>
       <c r="K8" s="5" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="10" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="B9" s="11" t="n">
         <v>46323</v>
@@ -2523,24 +2542,24 @@
         <v>3</v>
       </c>
       <c r="E9" s="5" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="F9" s="5" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="G9" s="6"/>
       <c r="H9" s="6"/>
       <c r="I9" s="14"/>
       <c r="J9" s="4" t="s">
-        <v>147</v>
+        <v>158</v>
       </c>
       <c r="K9" s="5" t="s">
-        <v>160</v>
+        <v>163</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="10" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="B10" s="11" t="n">
         <v>46326</v>
@@ -2553,24 +2572,24 @@
         <v>1</v>
       </c>
       <c r="E10" s="5" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="F10" s="5" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="G10" s="6"/>
       <c r="H10" s="6"/>
       <c r="I10" s="14"/>
       <c r="J10" s="4" t="s">
-        <v>147</v>
+        <v>158</v>
       </c>
       <c r="K10" s="5" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="10" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="B11" s="11" t="n">
         <v>46326</v>
@@ -2583,24 +2602,24 @@
         <v>3</v>
       </c>
       <c r="E11" s="5" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="F11" s="5" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="G11" s="6"/>
       <c r="H11" s="6"/>
       <c r="I11" s="14"/>
       <c r="J11" s="4" t="s">
-        <v>147</v>
+        <v>158</v>
       </c>
       <c r="K11" s="5" t="s">
-        <v>168</v>
+        <v>171</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="10" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="B12" s="11" t="n">
         <v>46330</v>
@@ -2613,24 +2632,24 @@
         <v>1</v>
       </c>
       <c r="E12" s="5" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="F12" s="5" t="s">
-        <v>171</v>
+        <v>174</v>
       </c>
       <c r="G12" s="6"/>
       <c r="H12" s="6"/>
       <c r="I12" s="14"/>
       <c r="J12" s="4" t="s">
-        <v>147</v>
+        <v>158</v>
       </c>
       <c r="K12" s="5" t="s">
-        <v>172</v>
+        <v>175</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="15" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="B13" s="16"/>
       <c r="C13" s="16"/>
@@ -2645,7 +2664,7 @@
       <c r="I13" s="16"/>
       <c r="J13" s="16"/>
       <c r="K13" s="17" t="s">
-        <v>174</v>
+        <v>177</v>
       </c>
     </row>
   </sheetData>
@@ -2692,12 +2711,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>175</v>
+        <v>178</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>176</v>
+        <v>179</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2705,25 +2724,25 @@
         <v>2</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>177</v>
+        <v>180</v>
       </c>
       <c r="C4" s="3" t="s">
         <v>130</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>178</v>
+        <v>181</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>179</v>
+        <v>182</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>180</v>
+        <v>183</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>181</v>
+        <v>184</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>182</v>
+        <v>185</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2731,49 +2750,49 @@
         <v>12</v>
       </c>
       <c r="B5" s="18" t="s">
-        <v>183</v>
+        <v>186</v>
       </c>
       <c r="C5" s="19" t="s">
-        <v>184</v>
+        <v>187</v>
       </c>
       <c r="D5" s="20" t="s">
         <v>60</v>
       </c>
       <c r="E5" s="20" t="s">
-        <v>185</v>
+        <v>188</v>
       </c>
       <c r="F5" s="20" t="s">
-        <v>186</v>
+        <v>189</v>
       </c>
       <c r="G5" s="20" t="s">
-        <v>187</v>
+        <v>190</v>
       </c>
       <c r="H5" s="20" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="18" t="s">
-        <v>188</v>
+        <v>191</v>
       </c>
       <c r="B6" s="18" t="s">
+        <v>192</v>
+      </c>
+      <c r="C6" s="19" t="s">
+        <v>172</v>
+      </c>
+      <c r="D6" s="20" t="s">
         <v>189</v>
       </c>
-      <c r="C6" s="19" t="s">
-        <v>169</v>
-      </c>
-      <c r="D6" s="20" t="s">
-        <v>186</v>
-      </c>
       <c r="E6" s="20" t="s">
-        <v>186</v>
+        <v>189</v>
       </c>
       <c r="F6" s="20" t="s">
-        <v>186</v>
+        <v>189</v>
       </c>
       <c r="G6" s="20"/>
       <c r="H6" s="20" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2781,25 +2800,25 @@
         <v>20</v>
       </c>
       <c r="B7" s="18" t="s">
-        <v>190</v>
+        <v>193</v>
       </c>
       <c r="C7" s="19" t="s">
-        <v>191</v>
+        <v>194</v>
       </c>
       <c r="D7" s="20" t="s">
-        <v>186</v>
+        <v>189</v>
       </c>
       <c r="E7" s="20" t="s">
-        <v>192</v>
+        <v>195</v>
       </c>
       <c r="F7" s="20" t="s">
-        <v>193</v>
+        <v>196</v>
       </c>
       <c r="G7" s="20" t="s">
-        <v>194</v>
+        <v>197</v>
       </c>
       <c r="H7" s="20" t="s">
-        <v>195</v>
+        <v>198</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2807,25 +2826,25 @@
         <v>29</v>
       </c>
       <c r="B8" s="18" t="s">
-        <v>196</v>
+        <v>199</v>
       </c>
       <c r="C8" s="19" t="s">
-        <v>197</v>
+        <v>200</v>
       </c>
       <c r="D8" s="20" t="s">
-        <v>198</v>
+        <v>201</v>
       </c>
       <c r="E8" s="20" t="s">
-        <v>199</v>
+        <v>202</v>
       </c>
       <c r="F8" s="20" t="s">
-        <v>200</v>
+        <v>203</v>
       </c>
       <c r="G8" s="20" t="s">
-        <v>201</v>
+        <v>204</v>
       </c>
       <c r="H8" s="20" t="s">
-        <v>202</v>
+        <v>205</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2833,22 +2852,22 @@
         <v>34</v>
       </c>
       <c r="B9" s="21" t="s">
-        <v>203</v>
+        <v>206</v>
       </c>
       <c r="C9" s="22" t="s">
-        <v>204</v>
+        <v>207</v>
       </c>
       <c r="D9" s="23" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
       <c r="E9" s="23" t="s">
-        <v>206</v>
+        <v>209</v>
       </c>
       <c r="F9" s="23" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
       <c r="G9" s="23" t="s">
-        <v>208</v>
+        <v>211</v>
       </c>
       <c r="H9" s="23" t="s">
         <v>139</v>
@@ -2856,25 +2875,25 @@
     </row>
     <row r="10" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="21" t="s">
-        <v>209</v>
+        <v>212</v>
       </c>
       <c r="B10" s="21" t="s">
-        <v>210</v>
+        <v>213</v>
       </c>
       <c r="C10" s="22" t="s">
         <v>139</v>
       </c>
       <c r="D10" s="23" t="s">
-        <v>211</v>
+        <v>214</v>
       </c>
       <c r="E10" s="23" t="s">
-        <v>212</v>
+        <v>215</v>
       </c>
       <c r="F10" s="23" t="s">
-        <v>213</v>
+        <v>216</v>
       </c>
       <c r="G10" s="23" t="s">
-        <v>214</v>
+        <v>217</v>
       </c>
       <c r="H10" s="23" t="s">
         <v>139</v>
@@ -2885,75 +2904,75 @@
         <v>41</v>
       </c>
       <c r="B11" s="21" t="s">
-        <v>215</v>
+        <v>218</v>
       </c>
       <c r="C11" s="22" t="s">
-        <v>216</v>
+        <v>219</v>
       </c>
       <c r="D11" s="23" t="s">
-        <v>217</v>
+        <v>220</v>
       </c>
       <c r="E11" s="23" t="s">
-        <v>218</v>
+        <v>221</v>
       </c>
       <c r="F11" s="23" t="s">
-        <v>219</v>
+        <v>222</v>
       </c>
       <c r="G11" s="23" t="s">
-        <v>220</v>
+        <v>223</v>
       </c>
       <c r="H11" s="23" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="21" t="s">
-        <v>221</v>
+        <v>224</v>
       </c>
       <c r="B12" s="21" t="s">
-        <v>183</v>
+        <v>186</v>
       </c>
       <c r="C12" s="22" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="D12" s="23" t="s">
-        <v>222</v>
+        <v>225</v>
       </c>
       <c r="E12" s="23" t="s">
-        <v>223</v>
+        <v>226</v>
       </c>
       <c r="F12" s="23" t="s">
-        <v>224</v>
+        <v>227</v>
       </c>
       <c r="G12" s="23" t="s">
-        <v>225</v>
+        <v>228</v>
       </c>
       <c r="H12" s="23" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="21" t="s">
-        <v>226</v>
+        <v>229</v>
       </c>
       <c r="B13" s="21" t="s">
-        <v>189</v>
+        <v>192</v>
       </c>
       <c r="C13" s="22" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="D13" s="23" t="s">
-        <v>227</v>
+        <v>230</v>
       </c>
       <c r="E13" s="23" t="s">
-        <v>228</v>
+        <v>231</v>
       </c>
       <c r="F13" s="23" t="s">
-        <v>229</v>
+        <v>232</v>
       </c>
       <c r="G13" s="23"/>
       <c r="H13" s="23" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2961,77 +2980,77 @@
         <v>48</v>
       </c>
       <c r="B14" s="21" t="s">
-        <v>190</v>
+        <v>193</v>
       </c>
       <c r="C14" s="22" t="s">
-        <v>230</v>
+        <v>233</v>
       </c>
       <c r="D14" s="23" t="s">
-        <v>231</v>
+        <v>234</v>
       </c>
       <c r="E14" s="23" t="s">
-        <v>232</v>
+        <v>235</v>
       </c>
       <c r="F14" s="23" t="s">
-        <v>233</v>
+        <v>236</v>
       </c>
       <c r="G14" s="23" t="s">
-        <v>234</v>
+        <v>237</v>
       </c>
       <c r="H14" s="23" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="21" t="s">
-        <v>235</v>
+        <v>238</v>
       </c>
       <c r="B15" s="21" t="s">
-        <v>196</v>
+        <v>199</v>
       </c>
       <c r="C15" s="22" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="D15" s="23" t="s">
-        <v>236</v>
+        <v>239</v>
       </c>
       <c r="E15" s="23" t="s">
-        <v>237</v>
+        <v>240</v>
       </c>
       <c r="F15" s="23" t="s">
-        <v>238</v>
+        <v>241</v>
       </c>
       <c r="G15" s="23" t="s">
-        <v>239</v>
+        <v>242</v>
       </c>
       <c r="H15" s="23" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="21" t="s">
-        <v>240</v>
+        <v>243</v>
       </c>
       <c r="B16" s="21" t="s">
-        <v>203</v>
+        <v>206</v>
       </c>
       <c r="C16" s="22" t="s">
-        <v>241</v>
+        <v>244</v>
       </c>
       <c r="D16" s="23" t="s">
-        <v>242</v>
+        <v>245</v>
       </c>
       <c r="E16" s="23" t="s">
-        <v>243</v>
+        <v>246</v>
       </c>
       <c r="F16" s="23" t="s">
-        <v>244</v>
+        <v>247</v>
       </c>
       <c r="G16" s="23" t="s">
-        <v>245</v>
+        <v>248</v>
       </c>
       <c r="H16" s="23" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3039,77 +3058,77 @@
         <v>54</v>
       </c>
       <c r="B17" s="21" t="s">
-        <v>210</v>
+        <v>213</v>
       </c>
       <c r="C17" s="22" t="s">
-        <v>246</v>
+        <v>249</v>
       </c>
       <c r="D17" s="23" t="s">
-        <v>247</v>
+        <v>250</v>
       </c>
       <c r="E17" s="23" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
       <c r="F17" s="23" t="s">
-        <v>249</v>
+        <v>252</v>
       </c>
       <c r="G17" s="8" t="s">
-        <v>250</v>
+        <v>253</v>
       </c>
       <c r="H17" s="23" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="21" t="s">
-        <v>252</v>
+        <v>255</v>
       </c>
       <c r="B18" s="21" t="s">
-        <v>215</v>
+        <v>218</v>
       </c>
       <c r="C18" s="22" t="s">
-        <v>253</v>
+        <v>256</v>
       </c>
       <c r="D18" s="23" t="s">
+        <v>257</v>
+      </c>
+      <c r="E18" s="23" t="s">
+        <v>258</v>
+      </c>
+      <c r="F18" s="23" t="s">
+        <v>259</v>
+      </c>
+      <c r="G18" s="23" t="s">
+        <v>260</v>
+      </c>
+      <c r="H18" s="23" t="s">
         <v>254</v>
-      </c>
-      <c r="E18" s="23" t="s">
-        <v>255</v>
-      </c>
-      <c r="F18" s="23" t="s">
-        <v>256</v>
-      </c>
-      <c r="G18" s="23" t="s">
-        <v>257</v>
-      </c>
-      <c r="H18" s="23" t="s">
-        <v>251</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="21" t="s">
-        <v>258</v>
+        <v>261</v>
       </c>
       <c r="B19" s="21" t="s">
-        <v>183</v>
+        <v>186</v>
       </c>
       <c r="C19" s="22" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
       <c r="D19" s="23" t="s">
-        <v>259</v>
+        <v>262</v>
       </c>
       <c r="E19" s="23" t="s">
-        <v>260</v>
+        <v>263</v>
       </c>
       <c r="F19" s="23" t="s">
-        <v>261</v>
+        <v>264</v>
       </c>
       <c r="G19" s="23" t="s">
-        <v>262</v>
+        <v>265</v>
       </c>
       <c r="H19" s="23" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3117,25 +3136,25 @@
         <v>62</v>
       </c>
       <c r="B20" s="21" t="s">
-        <v>189</v>
+        <v>192</v>
       </c>
       <c r="C20" s="22" t="s">
-        <v>263</v>
+        <v>266</v>
       </c>
       <c r="D20" s="23" t="s">
-        <v>264</v>
+        <v>267</v>
       </c>
       <c r="E20" s="23" t="s">
-        <v>265</v>
+        <v>268</v>
       </c>
       <c r="F20" s="23" t="s">
-        <v>266</v>
+        <v>269</v>
       </c>
       <c r="G20" s="23" t="s">
-        <v>267</v>
+        <v>270</v>
       </c>
       <c r="H20" s="23" t="s">
-        <v>268</v>
+        <v>271</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3143,25 +3162,25 @@
         <v>70</v>
       </c>
       <c r="B21" s="21" t="s">
-        <v>190</v>
+        <v>193</v>
       </c>
       <c r="C21" s="22" t="s">
-        <v>269</v>
+        <v>272</v>
       </c>
       <c r="D21" s="23" t="s">
-        <v>270</v>
+        <v>273</v>
       </c>
       <c r="E21" s="23" t="s">
-        <v>271</v>
+        <v>274</v>
       </c>
       <c r="F21" s="23" t="s">
-        <v>272</v>
+        <v>275</v>
       </c>
       <c r="G21" s="23" t="s">
-        <v>273</v>
+        <v>276</v>
       </c>
       <c r="H21" s="23" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3169,25 +3188,25 @@
         <v>85</v>
       </c>
       <c r="B22" s="21" t="s">
-        <v>196</v>
+        <v>199</v>
       </c>
       <c r="C22" s="22" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="D22" s="23" t="s">
-        <v>274</v>
+        <v>277</v>
       </c>
       <c r="E22" s="23" t="s">
-        <v>275</v>
+        <v>278</v>
       </c>
       <c r="F22" s="23" t="s">
-        <v>276</v>
+        <v>279</v>
       </c>
       <c r="G22" s="23" t="s">
-        <v>277</v>
+        <v>280</v>
       </c>
       <c r="H22" s="23" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3195,25 +3214,25 @@
         <v>91</v>
       </c>
       <c r="B23" s="18" t="s">
-        <v>203</v>
+        <v>206</v>
       </c>
       <c r="C23" s="19" t="s">
-        <v>278</v>
+        <v>281</v>
       </c>
       <c r="D23" s="20" t="s">
-        <v>279</v>
+        <v>282</v>
       </c>
       <c r="E23" s="20" t="s">
-        <v>280</v>
+        <v>283</v>
       </c>
       <c r="F23" s="20" t="s">
-        <v>281</v>
+        <v>284</v>
       </c>
       <c r="G23" s="20" t="s">
-        <v>282</v>
+        <v>285</v>
       </c>
       <c r="H23" s="20" t="s">
-        <v>195</v>
+        <v>198</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3221,25 +3240,25 @@
         <v>98</v>
       </c>
       <c r="B24" s="18" t="s">
-        <v>210</v>
+        <v>213</v>
       </c>
       <c r="C24" s="19" t="s">
-        <v>283</v>
+        <v>286</v>
       </c>
       <c r="D24" s="20" t="s">
-        <v>198</v>
+        <v>201</v>
       </c>
       <c r="E24" s="20" t="s">
-        <v>284</v>
+        <v>287</v>
       </c>
       <c r="F24" s="20" t="s">
-        <v>285</v>
+        <v>288</v>
       </c>
       <c r="G24" s="20" t="s">
-        <v>286</v>
+        <v>289</v>
       </c>
       <c r="H24" s="20" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3247,13 +3266,13 @@
         <v>99</v>
       </c>
       <c r="B25" s="18" t="s">
-        <v>215</v>
+        <v>218</v>
       </c>
       <c r="C25" s="19" t="s">
-        <v>287</v>
+        <v>290</v>
       </c>
       <c r="D25" s="20" t="s">
-        <v>288</v>
+        <v>291</v>
       </c>
       <c r="E25" s="20" t="s">
         <v>60</v>
@@ -3262,10 +3281,10 @@
         <v>60</v>
       </c>
       <c r="G25" s="20" t="s">
-        <v>289</v>
+        <v>292</v>
       </c>
       <c r="H25" s="20" t="s">
-        <v>290</v>
+        <v>293</v>
       </c>
     </row>
   </sheetData>
@@ -3297,26 +3316,26 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>291</v>
+        <v>294</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>292</v>
+        <v>295</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>293</v>
+        <v>296</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>294</v>
+        <v>297</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>295</v>
+        <v>298</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>296</v>
+        <v>299</v>
       </c>
       <c r="E4" s="3" t="s">
         <v>10</v>
@@ -3330,19 +3349,19 @@
         <v>1</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>297</v>
+        <v>300</v>
       </c>
       <c r="C5" s="4" t="s">
         <v>60</v>
       </c>
       <c r="D5" s="24" t="s">
-        <v>298</v>
+        <v>301</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>299</v>
+        <v>302</v>
       </c>
       <c r="F5" s="5" t="s">
-        <v>300</v>
+        <v>303</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3350,19 +3369,19 @@
         <v>2</v>
       </c>
       <c r="B6" s="5" t="s">
+        <v>304</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>305</v>
+      </c>
+      <c r="D6" s="24" t="s">
         <v>301</v>
       </c>
-      <c r="C6" s="4" t="s">
-        <v>302</v>
-      </c>
-      <c r="D6" s="24" t="s">
-        <v>298</v>
-      </c>
       <c r="E6" s="4" t="s">
-        <v>147</v>
+        <v>158</v>
       </c>
       <c r="F6" s="5" t="s">
-        <v>303</v>
+        <v>306</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3370,19 +3389,19 @@
         <v>3</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>304</v>
+        <v>307</v>
       </c>
       <c r="C7" s="4" t="s">
         <v>60</v>
       </c>
       <c r="D7" s="24" t="s">
-        <v>298</v>
+        <v>301</v>
       </c>
       <c r="E7" s="4" t="s">
-        <v>299</v>
+        <v>302</v>
       </c>
       <c r="F7" s="5" t="s">
-        <v>305</v>
+        <v>308</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3390,39 +3409,39 @@
         <v>4</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>306</v>
+        <v>309</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>307</v>
+        <v>60</v>
       </c>
       <c r="D8" s="24" t="s">
-        <v>298</v>
+        <v>301</v>
       </c>
       <c r="E8" s="4" t="s">
-        <v>147</v>
+        <v>302</v>
       </c>
       <c r="F8" s="5" t="s">
-        <v>308</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>310</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="n">
         <v>5</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>309</v>
+        <v>311</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>310</v>
+        <v>312</v>
       </c>
       <c r="D9" s="24" t="s">
-        <v>298</v>
+        <v>301</v>
       </c>
       <c r="E9" s="4" t="s">
-        <v>147</v>
+        <v>158</v>
       </c>
       <c r="F9" s="5" t="s">
-        <v>311</v>
+        <v>313</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3430,19 +3449,19 @@
         <v>6</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>312</v>
+        <v>314</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>313</v>
+        <v>60</v>
       </c>
       <c r="D10" s="24" t="s">
-        <v>298</v>
+        <v>301</v>
       </c>
       <c r="E10" s="4" t="s">
-        <v>147</v>
+        <v>302</v>
       </c>
       <c r="F10" s="5" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3450,19 +3469,19 @@
         <v>7</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="D11" s="24" t="s">
-        <v>298</v>
+        <v>301</v>
       </c>
       <c r="E11" s="4" t="s">
-        <v>147</v>
+        <v>158</v>
       </c>
       <c r="F11" s="5" t="s">
-        <v>314</v>
+        <v>318</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3470,19 +3489,19 @@
         <v>8</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>317</v>
+        <v>319</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>318</v>
+        <v>320</v>
       </c>
       <c r="D12" s="24" t="s">
-        <v>298</v>
+        <v>301</v>
       </c>
       <c r="E12" s="4" t="s">
-        <v>147</v>
+        <v>158</v>
       </c>
       <c r="F12" s="5" t="s">
-        <v>319</v>
+        <v>321</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3490,19 +3509,19 @@
         <v>9</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>320</v>
+        <v>322</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>321</v>
+        <v>323</v>
       </c>
       <c r="D13" s="4" t="s">
-        <v>322</v>
+        <v>324</v>
       </c>
       <c r="E13" s="4" t="s">
-        <v>147</v>
+        <v>158</v>
       </c>
       <c r="F13" s="5" t="s">
-        <v>314</v>
+        <v>318</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3510,19 +3529,19 @@
         <v>10</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>323</v>
+        <v>325</v>
       </c>
       <c r="C14" s="4" t="s">
+        <v>326</v>
+      </c>
+      <c r="D14" s="4" t="s">
         <v>324</v>
       </c>
-      <c r="D14" s="4" t="s">
-        <v>322</v>
-      </c>
       <c r="E14" s="4" t="s">
-        <v>147</v>
+        <v>158</v>
       </c>
       <c r="F14" s="5" t="s">
-        <v>325</v>
+        <v>327</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3530,19 +3549,19 @@
         <v>11</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
       <c r="D15" s="24" t="s">
-        <v>298</v>
+        <v>301</v>
       </c>
       <c r="E15" s="4" t="s">
-        <v>147</v>
+        <v>158</v>
       </c>
       <c r="F15" s="5" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3550,19 +3569,19 @@
         <v>12</v>
       </c>
       <c r="B16" s="5" t="s">
-        <v>329</v>
+        <v>331</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>313</v>
+        <v>332</v>
       </c>
       <c r="D16" s="4" t="s">
-        <v>322</v>
+        <v>324</v>
       </c>
       <c r="E16" s="4" t="s">
-        <v>147</v>
+        <v>158</v>
       </c>
       <c r="F16" s="5" t="s">
-        <v>330</v>
+        <v>333</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3570,19 +3589,19 @@
         <v>13</v>
       </c>
       <c r="B17" s="5" t="s">
-        <v>331</v>
+        <v>334</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="D17" s="4" t="s">
-        <v>332</v>
+        <v>335</v>
       </c>
       <c r="E17" s="4" t="s">
-        <v>147</v>
+        <v>158</v>
       </c>
       <c r="F17" s="5" t="s">
-        <v>333</v>
+        <v>336</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3590,19 +3609,19 @@
         <v>14</v>
       </c>
       <c r="B18" s="5" t="s">
-        <v>334</v>
+        <v>337</v>
       </c>
       <c r="C18" s="4" t="s">
+        <v>338</v>
+      </c>
+      <c r="D18" s="4" t="s">
         <v>335</v>
       </c>
-      <c r="D18" s="4" t="s">
-        <v>332</v>
-      </c>
       <c r="E18" s="4" t="s">
-        <v>147</v>
+        <v>158</v>
       </c>
       <c r="F18" s="5" t="s">
-        <v>336</v>
+        <v>339</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3610,19 +3629,19 @@
         <v>15</v>
       </c>
       <c r="B19" s="5" t="s">
-        <v>337</v>
+        <v>340</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>318</v>
+        <v>320</v>
       </c>
       <c r="D19" s="4" t="s">
-        <v>322</v>
+        <v>324</v>
       </c>
       <c r="E19" s="4" t="s">
-        <v>147</v>
+        <v>158</v>
       </c>
       <c r="F19" s="5" t="s">
-        <v>338</v>
+        <v>341</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3630,19 +3649,19 @@
         <v>16</v>
       </c>
       <c r="B20" s="5" t="s">
-        <v>339</v>
+        <v>342</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>321</v>
+        <v>323</v>
       </c>
       <c r="D20" s="4" t="s">
-        <v>322</v>
+        <v>324</v>
       </c>
       <c r="E20" s="4" t="s">
-        <v>147</v>
+        <v>158</v>
       </c>
       <c r="F20" s="5" t="s">
-        <v>340</v>
+        <v>343</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3650,19 +3669,19 @@
         <v>17</v>
       </c>
       <c r="B21" s="5" t="s">
-        <v>341</v>
+        <v>344</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>342</v>
+        <v>345</v>
       </c>
       <c r="D21" s="4" t="s">
-        <v>322</v>
+        <v>324</v>
       </c>
       <c r="E21" s="4" t="s">
-        <v>147</v>
+        <v>158</v>
       </c>
       <c r="F21" s="5" t="s">
-        <v>343</v>
+        <v>346</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3670,19 +3689,19 @@
         <v>18</v>
       </c>
       <c r="B22" s="5" t="s">
-        <v>344</v>
+        <v>347</v>
       </c>
       <c r="C22" s="4" t="s">
-        <v>342</v>
+        <v>345</v>
       </c>
       <c r="D22" s="4" t="s">
-        <v>322</v>
+        <v>324</v>
       </c>
       <c r="E22" s="4" t="s">
-        <v>147</v>
+        <v>158</v>
       </c>
       <c r="F22" s="5" t="s">
-        <v>345</v>
+        <v>348</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3690,19 +3709,19 @@
         <v>19</v>
       </c>
       <c r="B23" s="5" t="s">
-        <v>346</v>
+        <v>349</v>
       </c>
       <c r="C23" s="4" t="s">
-        <v>321</v>
+        <v>323</v>
       </c>
       <c r="D23" s="24" t="s">
-        <v>298</v>
+        <v>301</v>
       </c>
       <c r="E23" s="4" t="s">
-        <v>147</v>
+        <v>158</v>
       </c>
       <c r="F23" s="5" t="s">
-        <v>347</v>
+        <v>350</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3710,19 +3729,19 @@
         <v>20</v>
       </c>
       <c r="B24" s="5" t="s">
-        <v>348</v>
+        <v>351</v>
       </c>
       <c r="C24" s="4" t="s">
-        <v>321</v>
+        <v>323</v>
       </c>
       <c r="D24" s="4" t="s">
-        <v>322</v>
+        <v>324</v>
       </c>
       <c r="E24" s="4" t="s">
-        <v>147</v>
+        <v>158</v>
       </c>
       <c r="F24" s="5" t="s">
-        <v>349</v>
+        <v>352</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3730,19 +3749,19 @@
         <v>21</v>
       </c>
       <c r="B25" s="5" t="s">
-        <v>350</v>
+        <v>353</v>
       </c>
       <c r="C25" s="4" t="s">
+        <v>326</v>
+      </c>
+      <c r="D25" s="4" t="s">
         <v>324</v>
       </c>
-      <c r="D25" s="4" t="s">
-        <v>322</v>
-      </c>
       <c r="E25" s="4" t="s">
-        <v>147</v>
+        <v>158</v>
       </c>
       <c r="F25" s="5" t="s">
-        <v>351</v>
+        <v>354</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3750,19 +3769,19 @@
         <v>22</v>
       </c>
       <c r="B26" s="5" t="s">
-        <v>352</v>
+        <v>355</v>
       </c>
       <c r="C26" s="4" t="s">
         <v>60</v>
       </c>
       <c r="D26" s="4" t="s">
-        <v>332</v>
+        <v>335</v>
       </c>
       <c r="E26" s="4" t="s">
-        <v>299</v>
+        <v>302</v>
       </c>
       <c r="F26" s="5" t="s">
-        <v>353</v>
+        <v>356</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3770,19 +3789,19 @@
         <v>23</v>
       </c>
       <c r="B27" s="5" t="s">
-        <v>354</v>
+        <v>357</v>
       </c>
       <c r="C27" s="4" t="s">
-        <v>318</v>
+        <v>320</v>
       </c>
       <c r="D27" s="4" t="s">
-        <v>322</v>
+        <v>324</v>
       </c>
       <c r="E27" s="4" t="s">
-        <v>147</v>
+        <v>158</v>
       </c>
       <c r="F27" s="5" t="s">
-        <v>355</v>
+        <v>358</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3790,33 +3809,33 @@
         <v>24</v>
       </c>
       <c r="B28" s="5" t="s">
-        <v>356</v>
+        <v>359</v>
       </c>
       <c r="C28" s="4" t="s">
-        <v>310</v>
+        <v>312</v>
       </c>
       <c r="D28" s="4" t="s">
-        <v>332</v>
+        <v>335</v>
       </c>
       <c r="E28" s="4" t="s">
-        <v>147</v>
+        <v>158</v>
       </c>
       <c r="F28" s="5" t="s">
-        <v>357</v>
+        <v>360</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="15" t="s">
-        <v>358</v>
+        <v>361</v>
       </c>
       <c r="B30" s="25" t="n">
         <f aca="false">COUNTIF(E5:E28,"Concluído")</f>
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="15" t="s">
-        <v>359</v>
+        <v>362</v>
       </c>
       <c r="B31" s="25" t="n">
         <f aca="false">COUNTIF(E5:E28,"Em andamento")</f>
@@ -3825,20 +3844,20 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="15" t="s">
-        <v>360</v>
+        <v>363</v>
       </c>
       <c r="B32" s="25" t="n">
         <f aca="false">COUNTIF(E5:E28,"Pendente")</f>
-        <v>21</v>
+        <v>19</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="15" t="s">
-        <v>361</v>
+        <v>364</v>
       </c>
       <c r="B33" s="26" t="n">
         <f aca="false">IFERROR(B30/COUNTA(B5:B28),0)</f>
-        <v>0.125</v>
+        <v>0.208333333333333</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Confirm Baku-Tbilisi flight J2 8225 on 28/10
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FbPxpFjYDQnzNa7KTrLMWP
</commit_message>
<xml_diff>
--- a/Eurasia/Roteiro_Eurasia.xlsx
+++ b/Eurasia/Roteiro_Eurasia.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="549" uniqueCount="365">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="554" uniqueCount="368">
   <si>
     <t xml:space="preserve">Itinerário de Voos</t>
   </si>
@@ -190,405 +190,408 @@
     <t xml:space="preserve">28/10/2026</t>
   </si>
   <si>
-    <t xml:space="preserve">Baku (GYD) → Tbilisi (TBS)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AZAL (Azerbaijan Airlines)</t>
+    <t xml:space="preserve">Baku (GYD T1) → Tbilisi (TBS)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Azerbaijan Airlines (AZAL)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">J2 8225</t>
+  </si>
+  <si>
+    <t xml:space="preserve">20:50</t>
+  </si>
+  <si>
+    <t xml:space="preserve">22:00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">YQP6G9</t>
+  </si>
+  <si>
+    <t xml:space="preserve">31/10/2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tbilisi (TBS) → Atenas (ATH)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Aegean Airlines</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A3 897</t>
+  </si>
+  <si>
+    <t xml:space="preserve">06:00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">07:00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">9JCJ5F</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Claudio, Cristiano e Ney. Tarifa Light: só 1 volume (mala até 8 kg ou item pessoal).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">01/11/2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SKY express</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GQ 785</t>
+  </si>
+  <si>
+    <t xml:space="preserve">02:45</t>
+  </si>
+  <si>
+    <t xml:space="preserve">04:15</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HT190N</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Atenas (ATH) → Lisboa (LIS)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A3 (nº a confirmar)</t>
   </si>
   <si>
     <t xml:space="preserve">A confirmar</t>
   </si>
   <si>
-    <t xml:space="preserve">20:50</t>
-  </si>
-  <si>
-    <t xml:space="preserve">22:00</t>
+    <t xml:space="preserve">72MG3J</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ney. Claudio também precisa ir de Atenas a Lisboa neste dia (voo dele a confirmar).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lisboa (LIS) → Luanda (NBJ)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">653</t>
+  </si>
+  <si>
+    <t xml:space="preserve">22:35</t>
+  </si>
+  <si>
+    <t xml:space="preserve">06:30 (+1d)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Só Claudio. Precisa chegar de Atenas a Lisboa no mesmo dia.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">02/11/2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Luanda (NBJ) → São Paulo (GRU)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">747</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10:35</t>
+  </si>
+  <si>
+    <t xml:space="preserve">15:05</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Só Claudio.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">03/11/2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A3 720</t>
+  </si>
+  <si>
+    <t xml:space="preserve">08:35</t>
+  </si>
+  <si>
+    <t xml:space="preserve">11:05</t>
+  </si>
+  <si>
+    <t xml:space="preserve">XAISFZ</t>
+  </si>
+  <si>
+    <t xml:space="preserve">22:30</t>
+  </si>
+  <si>
+    <t xml:space="preserve">06:05 (+1d)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">04/11/2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">05/11/2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">São Paulo (CGH) → Brasília (BSB)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AD 6414</t>
+  </si>
+  <si>
+    <t xml:space="preserve">09:05</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10:55</t>
+  </si>
+  <si>
+    <t xml:space="preserve">13/11/2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Brasília (BSB) → Belo Horizonte (CNF)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gol</t>
+  </si>
+  <si>
+    <t xml:space="preserve">G3 1830</t>
+  </si>
+  <si>
+    <t xml:space="preserve">05:25</t>
+  </si>
+  <si>
+    <t xml:space="preserve">06:45</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LPSYTX</t>
+  </si>
+  <si>
+    <t xml:space="preserve">16/11/2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Belo Horizonte (CNF) → Brasília (BSB)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">G3 1309</t>
+  </si>
+  <si>
+    <t xml:space="preserve">09:45</t>
+  </si>
+  <si>
+    <t xml:space="preserve">11:00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">19/11/2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Brasília (BSB) → Rio de Janeiro (GIG)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LATAM</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LA 3245</t>
+  </si>
+  <si>
+    <t xml:space="preserve">19:30</t>
+  </si>
+  <si>
+    <t xml:space="preserve">21:15</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BVM-46V-8-26</t>
+  </si>
+  <si>
+    <t xml:space="preserve">24/11/2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rio de Janeiro (SDU) → Brasília (BSB)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">G3 1801</t>
+  </si>
+  <si>
+    <t xml:space="preserve">11:35</t>
+  </si>
+  <si>
+    <t xml:space="preserve">J2 8225 (28/10): tarifa Budget, sem bagagem despachada; 122,39 AZN. Check-in fecha 60 min antes. Meninos: confirmar se estão no mesmo voo.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hospedagem (hostels)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lilás = preencher após reservar. Noites e total calculados automaticamente. Lisboa não incluída.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cidade</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Check-in</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Check-out</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Noites</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chegada / saída</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Região sugerida</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hostel</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Valor total</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Observações</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Marraquexe</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chega 22:55 (20/10)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Medina, perto da Jemaa el-Fna</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Riad Hna Ben Saleh</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6552802435</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Reservado</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Riad Hna Ben Saleh, Derb Bouaanane, Ben Saleh nº 44, Medina. Quarto família, 4 adultos, café incluído. PAGAMENTO SÓ EM DINHEIRO (MAD). Não reembolsável. Avisar horário de chegada.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sai ~13:30 (22/10)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Segunda noite no mesmo riad. Pagamento em dinheiro (MAD).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Budapeste</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chega 20:30 (22/10) / sai ~09:45 (25/10)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Distrito VI (Terézváros)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Wombat's City Hostel</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Trip.com 20261022212925274204002979</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pago</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Wombat's City Hostel, Király u. 20, 1061 Budapeste. 1 cama, 3 noites. Check-in a partir das 14:00; check-out até 10:00. Valor: pagamento Trip.com de 22/10 (confirmar se é desta reserva).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Baku</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chega ~16:30 (25/10) / sai ~18:00 (28/10)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cidade Velha (Icherisheher) ou Nizami</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pendente</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pedir para guardar as mochilas no dia 28 até a saída para o aeroporto.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tbilisi (grupo, 4 pessoas)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chega ~22:30 (28/10) / meninos saem ~03:30 (31/10)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cidade Velha ou Sololaki</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Confirmar check-in tardio e saída de madrugada dos meninos (voo 06:00).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tbilisi (só Diego)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sai ~23:30 (31/10)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mesmo hostel</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cama em dormitório basta: garante descanso e banho até o voo das 02:45.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Atenas</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Meninos chegam 07:00 (31/10); Diego chega 04:15 (01/11) / Diego sai ~06:30 (03/11)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Monastiraki, Psyri ou Plaka</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Reserva a partir de 31/10 já cobre a chegada dos meninos e garante cama ao Diego de madrugada. Ney e Claudio saem em 01/11; confirmar data de Cristiano.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">São Paulo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chega 15:05 em GRU (04/11) / voo CGH 09:05 (05/11)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Perto de Congonhas (Moema, Campo Belo)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Só se não houver onde ficar.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Total</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Valores em moedas diferentes: não somados.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Roteiro: Lisboa, Marraquexe, Budapeste, Baku, Tbilisi, Kazbegi e Atenas (16/10 a 05/11/2026)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Verde = dias de passeio. Azul = dias de deslocamento. Amarelo = item ainda pendente.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dia</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Manhã</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tarde</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Noite</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Logística / Observações</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pernoite</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sex</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Brasília → São Paulo</t>
   </si>
   <si>
     <t xml:space="preserve">-</t>
   </si>
   <si>
-    <t xml:space="preserve">Pendente de compra</t>
-  </si>
-  <si>
-    <t xml:space="preserve">31/10/2026</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tbilisi (TBS) → Atenas (ATH)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Aegean Airlines</t>
-  </si>
-  <si>
-    <t xml:space="preserve">A3 897</t>
-  </si>
-  <si>
-    <t xml:space="preserve">06:00</t>
-  </si>
-  <si>
-    <t xml:space="preserve">07:00</t>
-  </si>
-  <si>
-    <t xml:space="preserve">9JCJ5F</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Claudio, Cristiano e Ney. Tarifa Light: só 1 volume (mala até 8 kg ou item pessoal).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">01/11/2026</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SKY express</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GQ 785</t>
-  </si>
-  <si>
-    <t xml:space="preserve">02:45</t>
-  </si>
-  <si>
-    <t xml:space="preserve">04:15</t>
-  </si>
-  <si>
-    <t xml:space="preserve">HT190N</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Atenas (ATH) → Lisboa (LIS)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">A3 (nº a confirmar)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">72MG3J</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ney. Claudio também precisa ir de Atenas a Lisboa neste dia (voo dele a confirmar).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Lisboa (LIS) → Luanda (NBJ)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">653</t>
-  </si>
-  <si>
-    <t xml:space="preserve">22:35</t>
-  </si>
-  <si>
-    <t xml:space="preserve">06:30 (+1d)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Só Claudio. Precisa chegar de Atenas a Lisboa no mesmo dia.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">02/11/2026</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Luanda (NBJ) → São Paulo (GRU)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">747</t>
-  </si>
-  <si>
-    <t xml:space="preserve">10:35</t>
-  </si>
-  <si>
-    <t xml:space="preserve">15:05</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Só Claudio.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">03/11/2026</t>
-  </si>
-  <si>
-    <t xml:space="preserve">A3 720</t>
-  </si>
-  <si>
-    <t xml:space="preserve">08:35</t>
-  </si>
-  <si>
-    <t xml:space="preserve">11:05</t>
-  </si>
-  <si>
-    <t xml:space="preserve">XAISFZ</t>
-  </si>
-  <si>
-    <t xml:space="preserve">22:30</t>
-  </si>
-  <si>
-    <t xml:space="preserve">06:05 (+1d)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">04/11/2026</t>
-  </si>
-  <si>
-    <t xml:space="preserve">05/11/2026</t>
-  </si>
-  <si>
-    <t xml:space="preserve">São Paulo (CGH) → Brasília (BSB)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AD 6414</t>
-  </si>
-  <si>
-    <t xml:space="preserve">09:05</t>
-  </si>
-  <si>
-    <t xml:space="preserve">10:55</t>
-  </si>
-  <si>
-    <t xml:space="preserve">13/11/2026</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Brasília (BSB) → Belo Horizonte (CNF)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Gol</t>
-  </si>
-  <si>
-    <t xml:space="preserve">G3 1830</t>
-  </si>
-  <si>
-    <t xml:space="preserve">05:25</t>
-  </si>
-  <si>
-    <t xml:space="preserve">06:45</t>
-  </si>
-  <si>
-    <t xml:space="preserve">LPSYTX</t>
-  </si>
-  <si>
-    <t xml:space="preserve">16/11/2026</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Belo Horizonte (CNF) → Brasília (BSB)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">G3 1309</t>
-  </si>
-  <si>
-    <t xml:space="preserve">09:45</t>
-  </si>
-  <si>
-    <t xml:space="preserve">11:00</t>
-  </si>
-  <si>
-    <t xml:space="preserve">19/11/2026</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Brasília (BSB) → Rio de Janeiro (GIG)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">LATAM</t>
-  </si>
-  <si>
-    <t xml:space="preserve">LA 3245</t>
-  </si>
-  <si>
-    <t xml:space="preserve">19:30</t>
-  </si>
-  <si>
-    <t xml:space="preserve">21:15</t>
-  </si>
-  <si>
-    <t xml:space="preserve">BVM-46V-8-26</t>
-  </si>
-  <si>
-    <t xml:space="preserve">24/11/2026</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Rio de Janeiro (SDU) → Brasília (BSB)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">G3 1801</t>
-  </si>
-  <si>
-    <t xml:space="preserve">11:35</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Voo pendente: cotação de R$ 407 (1 item pessoal + 1 mala de mão, sem despachada), direto, 1h10. Número do voo a confirmar na compra.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Hospedagem (hostels)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Lilás = preencher após reservar. Noites e total calculados automaticamente. Lisboa não incluída.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cidade</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Check-in</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Check-out</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Noites</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Chegada / saída</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Região sugerida</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Hostel</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Valor total</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Observações</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Marraquexe</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Chega 22:55 (20/10)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Medina, perto da Jemaa el-Fna</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Riad Hna Ben Saleh</t>
-  </si>
-  <si>
-    <t xml:space="preserve">6552802435</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Reservado</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Riad Hna Ben Saleh, Derb Bouaanane, Ben Saleh nº 44, Medina. Quarto família, 4 adultos, café incluído. PAGAMENTO SÓ EM DINHEIRO (MAD). Não reembolsável. Avisar horário de chegada.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sai ~13:30 (22/10)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Segunda noite no mesmo riad. Pagamento em dinheiro (MAD).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Budapeste</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Chega 20:30 (22/10) / sai ~09:45 (25/10)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Distrito VI (Terézváros)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Wombat's City Hostel</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Trip.com 20261022212925274204002979</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Pago</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Wombat's City Hostel, Király u. 20, 1061 Budapeste. 1 cama, 3 noites. Check-in a partir das 14:00; check-out até 10:00. Valor: pagamento Trip.com de 22/10 (confirmar se é desta reserva).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Baku</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Chega ~16:30 (25/10) / sai ~18:00 (28/10)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cidade Velha (Icherisheher) ou Nizami</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Pendente</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Pedir para guardar as mochilas no dia 28 até a saída para o aeroporto.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tbilisi (grupo, 4 pessoas)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Chega ~22:30 (28/10) / meninos saem ~03:30 (31/10)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cidade Velha ou Sololaki</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Confirmar check-in tardio e saída de madrugada dos meninos (voo 06:00).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tbilisi (só Diego)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sai ~23:30 (31/10)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Mesmo hostel</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cama em dormitório basta: garante descanso e banho até o voo das 02:45.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Atenas</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Meninos chegam 07:00 (31/10); Diego chega 04:15 (01/11) / Diego sai ~06:30 (03/11)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Monastiraki, Psyri ou Plaka</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Reserva a partir de 31/10 já cobre a chegada dos meninos e garante cama ao Diego de madrugada. Ney e Claudio saem em 01/11; confirmar data de Cristiano.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">São Paulo</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Chega 15:05 em GRU (04/11) / voo CGH 09:05 (05/11)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Perto de Congonhas (Moema, Campo Belo)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Só se não houver onde ficar.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Total</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Valores em moedas diferentes: não somados.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Roteiro: Lisboa, Marraquexe, Budapeste, Baku, Tbilisi, Kazbegi e Atenas (16/10 a 05/11/2026)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Verde = dias de passeio. Azul = dias de deslocamento. Amarelo = item ainda pendente.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Dia</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Manhã</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tarde</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Noite</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Logística / Observações</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Pernoite</t>
-  </si>
-  <si>
-    <t xml:space="preserve">sex</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Brasília → São Paulo</t>
-  </si>
-  <si>
     <t xml:space="preserve">Voo para São Paulo.</t>
   </si>
   <si>
@@ -784,7 +787,7 @@
     <t xml:space="preserve">Voo para Tbilisi.</t>
   </si>
   <si>
-    <t xml:space="preserve">AZAL GYD 20:50 → TBS 22:00 (PENDENTE DE COMPRA).</t>
+    <t xml:space="preserve">J2 8225 GYD (Terminal 1) 20:50 → TBS 22:00. Check-in fecha às 19:50.</t>
   </si>
   <si>
     <t xml:space="preserve">Tbilisi</t>
@@ -940,10 +943,16 @@
     <t xml:space="preserve">Comprar voo AZAL Baku → Tbilisi (28/10, 20:50)</t>
   </si>
   <si>
-    <t xml:space="preserve">Esta semana</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cotado a R$ 407 com mala de mão. Trem Baku–Tbilisi indisponível para quem entra com e-visa.</t>
+    <t xml:space="preserve">Diego: J2 8225, YQP6G9, 122,39 AZN.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Confirmar voo dos meninos Baku → Tbilisi (28/10)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Até 26/10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ideal no mesmo J2 8225 das 20:50.</t>
   </si>
   <si>
     <t xml:space="preserve">Hospedagem Marraquexe 20 a 21/10</t>
@@ -1201,7 +1210,7 @@
       <charset val="1"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1217,12 +1226,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFEDE7F6"/>
-        <bgColor rgb="FFF2F2F2"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFF2CC"/>
         <bgColor rgb="FFF2F2F2"/>
       </patternFill>
     </fill>
@@ -1294,7 +1297,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="24">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1323,18 +1326,6 @@
       <alignment horizontal="center" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="164" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1355,16 +1346,28 @@
       <alignment horizontal="center" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="5" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="7" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
@@ -1376,18 +1379,6 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="7" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1905,84 +1896,84 @@
       <c r="J10" s="5"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="7" t="s">
+      <c r="A11" s="4" t="s">
         <v>54</v>
       </c>
-      <c r="B11" s="8" t="s">
+      <c r="B11" s="5" t="s">
         <v>55</v>
       </c>
-      <c r="C11" s="8" t="s">
+      <c r="C11" s="5" t="s">
         <v>56</v>
       </c>
-      <c r="D11" s="7" t="s">
+      <c r="D11" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="E11" s="7" t="s">
+      <c r="E11" s="4" t="s">
         <v>58</v>
       </c>
-      <c r="F11" s="7" t="s">
+      <c r="F11" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="G11" s="7" t="s">
+      <c r="G11" s="4" t="s">
         <v>60</v>
       </c>
       <c r="H11" s="6"/>
-      <c r="I11" s="9" t="s">
-        <v>61</v>
+      <c r="I11" s="4" t="s">
+        <v>19</v>
       </c>
       <c r="J11" s="5"/>
     </row>
     <row r="12" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="B12" s="5" t="s">
         <v>62</v>
       </c>
-      <c r="B12" s="5" t="s">
+      <c r="C12" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="C12" s="5" t="s">
+      <c r="D12" s="4" t="s">
         <v>64</v>
       </c>
-      <c r="D12" s="4" t="s">
+      <c r="E12" s="4" t="s">
         <v>65</v>
       </c>
-      <c r="E12" s="4" t="s">
+      <c r="F12" s="4" t="s">
         <v>66</v>
-      </c>
-      <c r="F12" s="4" t="s">
-        <v>67</v>
       </c>
       <c r="G12" s="4"/>
       <c r="H12" s="6" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="I12" s="4" t="s">
         <v>19</v>
       </c>
       <c r="J12" s="5" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="4" t="s">
+        <v>69</v>
+      </c>
+      <c r="B13" s="5" t="s">
+        <v>62</v>
+      </c>
+      <c r="C13" s="5" t="s">
         <v>70</v>
       </c>
-      <c r="B13" s="5" t="s">
-        <v>63</v>
-      </c>
-      <c r="C13" s="5" t="s">
+      <c r="D13" s="4" t="s">
         <v>71</v>
       </c>
-      <c r="D13" s="4" t="s">
+      <c r="E13" s="4" t="s">
         <v>72</v>
       </c>
-      <c r="E13" s="4" t="s">
+      <c r="F13" s="4" t="s">
         <v>73</v>
       </c>
-      <c r="F13" s="4" t="s">
+      <c r="G13" s="4" t="s">
         <v>74</v>
-      </c>
-      <c r="G13" s="4" t="s">
-        <v>75</v>
       </c>
       <c r="H13" s="6"/>
       <c r="I13" s="4" t="s">
@@ -1992,22 +1983,22 @@
     </row>
     <row r="14" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="4" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B14" s="5" t="s">
+        <v>75</v>
+      </c>
+      <c r="C14" s="5" t="s">
+        <v>63</v>
+      </c>
+      <c r="D14" s="4" t="s">
         <v>76</v>
       </c>
-      <c r="C14" s="5" t="s">
-        <v>64</v>
-      </c>
-      <c r="D14" s="4" t="s">
+      <c r="E14" s="4" t="s">
         <v>77</v>
       </c>
-      <c r="E14" s="4" t="s">
-        <v>57</v>
-      </c>
       <c r="F14" s="4" t="s">
-        <v>57</v>
+        <v>77</v>
       </c>
       <c r="G14" s="4"/>
       <c r="H14" s="6" t="s">
@@ -2022,7 +2013,7 @@
     </row>
     <row r="15" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="4" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B15" s="5" t="s">
         <v>80</v>
@@ -2085,10 +2076,10 @@
         <v>91</v>
       </c>
       <c r="B17" s="5" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C17" s="5" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="D17" s="4" t="s">
         <v>92</v>
@@ -2392,13 +2383,13 @@
       </c>
     </row>
     <row r="5" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="10" t="s">
+      <c r="A5" s="7" t="s">
         <v>139</v>
       </c>
-      <c r="B5" s="11" t="n">
+      <c r="B5" s="8" t="n">
         <v>46315</v>
       </c>
-      <c r="C5" s="11" t="n">
+      <c r="C5" s="8" t="n">
         <v>46316</v>
       </c>
       <c r="D5" s="4" t="n">
@@ -2417,24 +2408,24 @@
       <c r="H5" s="6" t="s">
         <v>143</v>
       </c>
-      <c r="I5" s="12" t="n">
+      <c r="I5" s="9" t="n">
         <v>80</v>
       </c>
       <c r="J5" s="4" t="s">
         <v>144</v>
       </c>
-      <c r="K5" s="13" t="s">
+      <c r="K5" s="10" t="s">
         <v>145</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="10" t="s">
+      <c r="A6" s="7" t="s">
         <v>139</v>
       </c>
-      <c r="B6" s="11" t="n">
+      <c r="B6" s="8" t="n">
         <v>46316</v>
       </c>
-      <c r="C6" s="11" t="n">
+      <c r="C6" s="8" t="n">
         <v>46317</v>
       </c>
       <c r="D6" s="4" t="n">
@@ -2451,7 +2442,7 @@
         <v>142</v>
       </c>
       <c r="H6" s="6"/>
-      <c r="I6" s="12" t="n">
+      <c r="I6" s="9" t="n">
         <v>80</v>
       </c>
       <c r="J6" s="4" t="s">
@@ -2462,13 +2453,13 @@
       </c>
     </row>
     <row r="7" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="10" t="s">
+      <c r="A7" s="7" t="s">
         <v>148</v>
       </c>
-      <c r="B7" s="11" t="n">
+      <c r="B7" s="8" t="n">
         <v>46317</v>
       </c>
-      <c r="C7" s="11" t="n">
+      <c r="C7" s="8" t="n">
         <v>46320</v>
       </c>
       <c r="D7" s="4" t="n">
@@ -2487,7 +2478,7 @@
       <c r="H7" s="6" t="s">
         <v>152</v>
       </c>
-      <c r="I7" s="14" t="n">
+      <c r="I7" s="11" t="n">
         <v>840.92</v>
       </c>
       <c r="J7" s="4" t="s">
@@ -2498,13 +2489,13 @@
       </c>
     </row>
     <row r="8" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="10" t="s">
+      <c r="A8" s="7" t="s">
         <v>155</v>
       </c>
-      <c r="B8" s="11" t="n">
+      <c r="B8" s="8" t="n">
         <v>46320</v>
       </c>
-      <c r="C8" s="11" t="n">
+      <c r="C8" s="8" t="n">
         <v>46323</v>
       </c>
       <c r="D8" s="4" t="n">
@@ -2519,7 +2510,7 @@
       </c>
       <c r="G8" s="6"/>
       <c r="H8" s="6"/>
-      <c r="I8" s="14"/>
+      <c r="I8" s="11"/>
       <c r="J8" s="4" t="s">
         <v>158</v>
       </c>
@@ -2528,13 +2519,13 @@
       </c>
     </row>
     <row r="9" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="10" t="s">
+      <c r="A9" s="7" t="s">
         <v>160</v>
       </c>
-      <c r="B9" s="11" t="n">
+      <c r="B9" s="8" t="n">
         <v>46323</v>
       </c>
-      <c r="C9" s="11" t="n">
+      <c r="C9" s="8" t="n">
         <v>46326</v>
       </c>
       <c r="D9" s="4" t="n">
@@ -2549,7 +2540,7 @@
       </c>
       <c r="G9" s="6"/>
       <c r="H9" s="6"/>
-      <c r="I9" s="14"/>
+      <c r="I9" s="11"/>
       <c r="J9" s="4" t="s">
         <v>158</v>
       </c>
@@ -2558,13 +2549,13 @@
       </c>
     </row>
     <row r="10" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="10" t="s">
+      <c r="A10" s="7" t="s">
         <v>164</v>
       </c>
-      <c r="B10" s="11" t="n">
+      <c r="B10" s="8" t="n">
         <v>46326</v>
       </c>
-      <c r="C10" s="11" t="n">
+      <c r="C10" s="8" t="n">
         <v>46327</v>
       </c>
       <c r="D10" s="4" t="n">
@@ -2579,7 +2570,7 @@
       </c>
       <c r="G10" s="6"/>
       <c r="H10" s="6"/>
-      <c r="I10" s="14"/>
+      <c r="I10" s="11"/>
       <c r="J10" s="4" t="s">
         <v>158</v>
       </c>
@@ -2588,13 +2579,13 @@
       </c>
     </row>
     <row r="11" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="10" t="s">
+      <c r="A11" s="7" t="s">
         <v>168</v>
       </c>
-      <c r="B11" s="11" t="n">
+      <c r="B11" s="8" t="n">
         <v>46326</v>
       </c>
-      <c r="C11" s="11" t="n">
+      <c r="C11" s="8" t="n">
         <v>46329</v>
       </c>
       <c r="D11" s="4" t="n">
@@ -2609,7 +2600,7 @@
       </c>
       <c r="G11" s="6"/>
       <c r="H11" s="6"/>
-      <c r="I11" s="14"/>
+      <c r="I11" s="11"/>
       <c r="J11" s="4" t="s">
         <v>158</v>
       </c>
@@ -2618,13 +2609,13 @@
       </c>
     </row>
     <row r="12" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="10" t="s">
+      <c r="A12" s="7" t="s">
         <v>172</v>
       </c>
-      <c r="B12" s="11" t="n">
+      <c r="B12" s="8" t="n">
         <v>46330</v>
       </c>
-      <c r="C12" s="11" t="n">
+      <c r="C12" s="8" t="n">
         <v>46331</v>
       </c>
       <c r="D12" s="4" t="n">
@@ -2639,7 +2630,7 @@
       </c>
       <c r="G12" s="6"/>
       <c r="H12" s="6"/>
-      <c r="I12" s="14"/>
+      <c r="I12" s="11"/>
       <c r="J12" s="4" t="s">
         <v>158</v>
       </c>
@@ -2648,22 +2639,22 @@
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="15" t="s">
+      <c r="A13" s="12" t="s">
         <v>176</v>
       </c>
-      <c r="B13" s="16"/>
-      <c r="C13" s="16"/>
-      <c r="D13" s="15" t="n">
+      <c r="B13" s="13"/>
+      <c r="C13" s="13"/>
+      <c r="D13" s="12" t="n">
         <f aca="false">SUM(D5:D12)</f>
         <v>16</v>
       </c>
-      <c r="E13" s="16"/>
-      <c r="F13" s="16"/>
-      <c r="G13" s="16"/>
-      <c r="H13" s="16"/>
-      <c r="I13" s="16"/>
-      <c r="J13" s="16"/>
-      <c r="K13" s="17" t="s">
+      <c r="E13" s="13"/>
+      <c r="F13" s="13"/>
+      <c r="G13" s="13"/>
+      <c r="H13" s="13"/>
+      <c r="I13" s="13"/>
+      <c r="J13" s="13"/>
+      <c r="K13" s="14" t="s">
         <v>177</v>
       </c>
     </row>
@@ -2746,545 +2737,545 @@
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="18" t="s">
+      <c r="A5" s="15" t="s">
         <v>12</v>
       </c>
-      <c r="B5" s="18" t="s">
+      <c r="B5" s="15" t="s">
         <v>186</v>
       </c>
-      <c r="C5" s="19" t="s">
+      <c r="C5" s="16" t="s">
         <v>187</v>
       </c>
-      <c r="D5" s="20" t="s">
-        <v>60</v>
-      </c>
-      <c r="E5" s="20" t="s">
+      <c r="D5" s="17" t="s">
         <v>188</v>
       </c>
-      <c r="F5" s="20" t="s">
+      <c r="E5" s="17" t="s">
         <v>189</v>
       </c>
-      <c r="G5" s="20" t="s">
+      <c r="F5" s="17" t="s">
         <v>190</v>
       </c>
-      <c r="H5" s="20" t="s">
+      <c r="G5" s="17" t="s">
+        <v>191</v>
+      </c>
+      <c r="H5" s="17" t="s">
         <v>172</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="18" t="s">
-        <v>191</v>
-      </c>
-      <c r="B6" s="18" t="s">
+      <c r="A6" s="15" t="s">
         <v>192</v>
       </c>
-      <c r="C6" s="19" t="s">
+      <c r="B6" s="15" t="s">
+        <v>193</v>
+      </c>
+      <c r="C6" s="16" t="s">
         <v>172</v>
       </c>
-      <c r="D6" s="20" t="s">
-        <v>189</v>
-      </c>
-      <c r="E6" s="20" t="s">
-        <v>189</v>
-      </c>
-      <c r="F6" s="20" t="s">
-        <v>189</v>
-      </c>
-      <c r="G6" s="20"/>
-      <c r="H6" s="20" t="s">
+      <c r="D6" s="17" t="s">
+        <v>190</v>
+      </c>
+      <c r="E6" s="17" t="s">
+        <v>190</v>
+      </c>
+      <c r="F6" s="17" t="s">
+        <v>190</v>
+      </c>
+      <c r="G6" s="17"/>
+      <c r="H6" s="17" t="s">
         <v>172</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="18" t="s">
+      <c r="A7" s="15" t="s">
         <v>20</v>
       </c>
-      <c r="B7" s="18" t="s">
+      <c r="B7" s="15" t="s">
+        <v>194</v>
+      </c>
+      <c r="C7" s="16" t="s">
+        <v>195</v>
+      </c>
+      <c r="D7" s="17" t="s">
+        <v>190</v>
+      </c>
+      <c r="E7" s="17" t="s">
+        <v>196</v>
+      </c>
+      <c r="F7" s="17" t="s">
+        <v>197</v>
+      </c>
+      <c r="G7" s="17" t="s">
+        <v>198</v>
+      </c>
+      <c r="H7" s="17" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="15" t="s">
+        <v>29</v>
+      </c>
+      <c r="B8" s="15" t="s">
+        <v>200</v>
+      </c>
+      <c r="C8" s="16" t="s">
+        <v>201</v>
+      </c>
+      <c r="D8" s="17" t="s">
+        <v>202</v>
+      </c>
+      <c r="E8" s="17" t="s">
+        <v>203</v>
+      </c>
+      <c r="F8" s="17" t="s">
+        <v>204</v>
+      </c>
+      <c r="G8" s="17" t="s">
+        <v>205</v>
+      </c>
+      <c r="H8" s="17" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="18" t="s">
+        <v>34</v>
+      </c>
+      <c r="B9" s="18" t="s">
+        <v>207</v>
+      </c>
+      <c r="C9" s="19" t="s">
+        <v>208</v>
+      </c>
+      <c r="D9" s="20" t="s">
+        <v>209</v>
+      </c>
+      <c r="E9" s="20" t="s">
+        <v>210</v>
+      </c>
+      <c r="F9" s="20" t="s">
+        <v>211</v>
+      </c>
+      <c r="G9" s="20" t="s">
+        <v>212</v>
+      </c>
+      <c r="H9" s="20" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="18" t="s">
+        <v>213</v>
+      </c>
+      <c r="B10" s="18" t="s">
+        <v>214</v>
+      </c>
+      <c r="C10" s="19" t="s">
+        <v>139</v>
+      </c>
+      <c r="D10" s="20" t="s">
+        <v>215</v>
+      </c>
+      <c r="E10" s="20" t="s">
+        <v>216</v>
+      </c>
+      <c r="F10" s="20" t="s">
+        <v>217</v>
+      </c>
+      <c r="G10" s="20" t="s">
+        <v>218</v>
+      </c>
+      <c r="H10" s="20" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="18" t="s">
+        <v>41</v>
+      </c>
+      <c r="B11" s="18" t="s">
+        <v>219</v>
+      </c>
+      <c r="C11" s="19" t="s">
+        <v>220</v>
+      </c>
+      <c r="D11" s="20" t="s">
+        <v>221</v>
+      </c>
+      <c r="E11" s="20" t="s">
+        <v>222</v>
+      </c>
+      <c r="F11" s="20" t="s">
+        <v>223</v>
+      </c>
+      <c r="G11" s="20" t="s">
+        <v>224</v>
+      </c>
+      <c r="H11" s="20" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="18" t="s">
+        <v>225</v>
+      </c>
+      <c r="B12" s="18" t="s">
+        <v>186</v>
+      </c>
+      <c r="C12" s="19" t="s">
+        <v>148</v>
+      </c>
+      <c r="D12" s="20" t="s">
+        <v>226</v>
+      </c>
+      <c r="E12" s="20" t="s">
+        <v>227</v>
+      </c>
+      <c r="F12" s="20" t="s">
+        <v>228</v>
+      </c>
+      <c r="G12" s="20" t="s">
+        <v>229</v>
+      </c>
+      <c r="H12" s="20" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="18" t="s">
+        <v>230</v>
+      </c>
+      <c r="B13" s="18" t="s">
         <v>193</v>
       </c>
-      <c r="C7" s="19" t="s">
+      <c r="C13" s="19" t="s">
+        <v>148</v>
+      </c>
+      <c r="D13" s="20" t="s">
+        <v>231</v>
+      </c>
+      <c r="E13" s="20" t="s">
+        <v>232</v>
+      </c>
+      <c r="F13" s="20" t="s">
+        <v>233</v>
+      </c>
+      <c r="G13" s="20"/>
+      <c r="H13" s="20" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="18" t="s">
+        <v>48</v>
+      </c>
+      <c r="B14" s="18" t="s">
         <v>194</v>
       </c>
-      <c r="D7" s="20" t="s">
-        <v>189</v>
-      </c>
-      <c r="E7" s="20" t="s">
-        <v>195</v>
-      </c>
-      <c r="F7" s="20" t="s">
-        <v>196</v>
-      </c>
-      <c r="G7" s="20" t="s">
-        <v>197</v>
-      </c>
-      <c r="H7" s="20" t="s">
-        <v>198</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="18" t="s">
-        <v>29</v>
-      </c>
-      <c r="B8" s="18" t="s">
+      <c r="C14" s="19" t="s">
+        <v>234</v>
+      </c>
+      <c r="D14" s="20" t="s">
+        <v>235</v>
+      </c>
+      <c r="E14" s="20" t="s">
+        <v>236</v>
+      </c>
+      <c r="F14" s="20" t="s">
+        <v>237</v>
+      </c>
+      <c r="G14" s="20" t="s">
+        <v>238</v>
+      </c>
+      <c r="H14" s="20" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="18" t="s">
+        <v>239</v>
+      </c>
+      <c r="B15" s="18" t="s">
+        <v>200</v>
+      </c>
+      <c r="C15" s="19" t="s">
+        <v>155</v>
+      </c>
+      <c r="D15" s="20" t="s">
+        <v>240</v>
+      </c>
+      <c r="E15" s="20" t="s">
+        <v>241</v>
+      </c>
+      <c r="F15" s="20" t="s">
+        <v>242</v>
+      </c>
+      <c r="G15" s="20" t="s">
+        <v>243</v>
+      </c>
+      <c r="H15" s="20" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="18" t="s">
+        <v>244</v>
+      </c>
+      <c r="B16" s="18" t="s">
+        <v>207</v>
+      </c>
+      <c r="C16" s="19" t="s">
+        <v>245</v>
+      </c>
+      <c r="D16" s="20" t="s">
+        <v>246</v>
+      </c>
+      <c r="E16" s="20" t="s">
+        <v>247</v>
+      </c>
+      <c r="F16" s="20" t="s">
+        <v>248</v>
+      </c>
+      <c r="G16" s="20" t="s">
+        <v>249</v>
+      </c>
+      <c r="H16" s="20" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="18" t="s">
+        <v>54</v>
+      </c>
+      <c r="B17" s="18" t="s">
+        <v>214</v>
+      </c>
+      <c r="C17" s="19" t="s">
+        <v>250</v>
+      </c>
+      <c r="D17" s="20" t="s">
+        <v>251</v>
+      </c>
+      <c r="E17" s="20" t="s">
+        <v>252</v>
+      </c>
+      <c r="F17" s="20" t="s">
+        <v>253</v>
+      </c>
+      <c r="G17" s="20" t="s">
+        <v>254</v>
+      </c>
+      <c r="H17" s="20" t="s">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="18" t="s">
+        <v>256</v>
+      </c>
+      <c r="B18" s="18" t="s">
+        <v>219</v>
+      </c>
+      <c r="C18" s="19" t="s">
+        <v>257</v>
+      </c>
+      <c r="D18" s="20" t="s">
+        <v>258</v>
+      </c>
+      <c r="E18" s="20" t="s">
+        <v>259</v>
+      </c>
+      <c r="F18" s="20" t="s">
+        <v>260</v>
+      </c>
+      <c r="G18" s="20" t="s">
+        <v>261</v>
+      </c>
+      <c r="H18" s="20" t="s">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="18" t="s">
+        <v>262</v>
+      </c>
+      <c r="B19" s="18" t="s">
+        <v>186</v>
+      </c>
+      <c r="C19" s="19" t="s">
+        <v>255</v>
+      </c>
+      <c r="D19" s="20" t="s">
+        <v>263</v>
+      </c>
+      <c r="E19" s="20" t="s">
+        <v>264</v>
+      </c>
+      <c r="F19" s="20" t="s">
+        <v>265</v>
+      </c>
+      <c r="G19" s="20" t="s">
+        <v>266</v>
+      </c>
+      <c r="H19" s="20" t="s">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="18" t="s">
+        <v>61</v>
+      </c>
+      <c r="B20" s="18" t="s">
+        <v>193</v>
+      </c>
+      <c r="C20" s="19" t="s">
+        <v>267</v>
+      </c>
+      <c r="D20" s="20" t="s">
+        <v>268</v>
+      </c>
+      <c r="E20" s="20" t="s">
+        <v>269</v>
+      </c>
+      <c r="F20" s="20" t="s">
+        <v>270</v>
+      </c>
+      <c r="G20" s="20" t="s">
+        <v>271</v>
+      </c>
+      <c r="H20" s="20" t="s">
+        <v>272</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="18" t="s">
+        <v>69</v>
+      </c>
+      <c r="B21" s="18" t="s">
+        <v>194</v>
+      </c>
+      <c r="C21" s="19" t="s">
+        <v>273</v>
+      </c>
+      <c r="D21" s="20" t="s">
+        <v>274</v>
+      </c>
+      <c r="E21" s="20" t="s">
+        <v>275</v>
+      </c>
+      <c r="F21" s="20" t="s">
+        <v>276</v>
+      </c>
+      <c r="G21" s="20" t="s">
+        <v>277</v>
+      </c>
+      <c r="H21" s="20" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="18" t="s">
+        <v>85</v>
+      </c>
+      <c r="B22" s="18" t="s">
+        <v>200</v>
+      </c>
+      <c r="C22" s="19" t="s">
+        <v>168</v>
+      </c>
+      <c r="D22" s="20" t="s">
+        <v>278</v>
+      </c>
+      <c r="E22" s="20" t="s">
+        <v>279</v>
+      </c>
+      <c r="F22" s="20" t="s">
+        <v>280</v>
+      </c>
+      <c r="G22" s="20" t="s">
+        <v>281</v>
+      </c>
+      <c r="H22" s="20" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="15" t="s">
+        <v>91</v>
+      </c>
+      <c r="B23" s="15" t="s">
+        <v>207</v>
+      </c>
+      <c r="C23" s="16" t="s">
+        <v>282</v>
+      </c>
+      <c r="D23" s="17" t="s">
+        <v>283</v>
+      </c>
+      <c r="E23" s="17" t="s">
+        <v>284</v>
+      </c>
+      <c r="F23" s="17" t="s">
+        <v>285</v>
+      </c>
+      <c r="G23" s="17" t="s">
+        <v>286</v>
+      </c>
+      <c r="H23" s="17" t="s">
         <v>199</v>
       </c>
-      <c r="C8" s="19" t="s">
-        <v>200</v>
-      </c>
-      <c r="D8" s="20" t="s">
-        <v>201</v>
-      </c>
-      <c r="E8" s="20" t="s">
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="15" t="s">
+        <v>98</v>
+      </c>
+      <c r="B24" s="15" t="s">
+        <v>214</v>
+      </c>
+      <c r="C24" s="16" t="s">
+        <v>287</v>
+      </c>
+      <c r="D24" s="17" t="s">
         <v>202</v>
       </c>
-      <c r="F8" s="20" t="s">
-        <v>203</v>
-      </c>
-      <c r="G8" s="20" t="s">
-        <v>204</v>
-      </c>
-      <c r="H8" s="20" t="s">
-        <v>205</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="21" t="s">
-        <v>34</v>
-      </c>
-      <c r="B9" s="21" t="s">
-        <v>206</v>
-      </c>
-      <c r="C9" s="22" t="s">
-        <v>207</v>
-      </c>
-      <c r="D9" s="23" t="s">
-        <v>208</v>
-      </c>
-      <c r="E9" s="23" t="s">
-        <v>209</v>
-      </c>
-      <c r="F9" s="23" t="s">
-        <v>210</v>
-      </c>
-      <c r="G9" s="23" t="s">
-        <v>211</v>
-      </c>
-      <c r="H9" s="23" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="21" t="s">
-        <v>212</v>
-      </c>
-      <c r="B10" s="21" t="s">
-        <v>213</v>
-      </c>
-      <c r="C10" s="22" t="s">
-        <v>139</v>
-      </c>
-      <c r="D10" s="23" t="s">
-        <v>214</v>
-      </c>
-      <c r="E10" s="23" t="s">
-        <v>215</v>
-      </c>
-      <c r="F10" s="23" t="s">
-        <v>216</v>
-      </c>
-      <c r="G10" s="23" t="s">
-        <v>217</v>
-      </c>
-      <c r="H10" s="23" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="21" t="s">
-        <v>41</v>
-      </c>
-      <c r="B11" s="21" t="s">
-        <v>218</v>
-      </c>
-      <c r="C11" s="22" t="s">
+      <c r="E24" s="17" t="s">
+        <v>288</v>
+      </c>
+      <c r="F24" s="17" t="s">
+        <v>289</v>
+      </c>
+      <c r="G24" s="17" t="s">
+        <v>290</v>
+      </c>
+      <c r="H24" s="17" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="15" t="s">
+        <v>99</v>
+      </c>
+      <c r="B25" s="15" t="s">
         <v>219</v>
       </c>
-      <c r="D11" s="23" t="s">
-        <v>220</v>
-      </c>
-      <c r="E11" s="23" t="s">
-        <v>221</v>
-      </c>
-      <c r="F11" s="23" t="s">
-        <v>222</v>
-      </c>
-      <c r="G11" s="23" t="s">
-        <v>223</v>
-      </c>
-      <c r="H11" s="23" t="s">
-        <v>148</v>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="21" t="s">
-        <v>224</v>
-      </c>
-      <c r="B12" s="21" t="s">
-        <v>186</v>
-      </c>
-      <c r="C12" s="22" t="s">
-        <v>148</v>
-      </c>
-      <c r="D12" s="23" t="s">
-        <v>225</v>
-      </c>
-      <c r="E12" s="23" t="s">
-        <v>226</v>
-      </c>
-      <c r="F12" s="23" t="s">
-        <v>227</v>
-      </c>
-      <c r="G12" s="23" t="s">
-        <v>228</v>
-      </c>
-      <c r="H12" s="23" t="s">
-        <v>148</v>
-      </c>
-    </row>
-    <row r="13" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="21" t="s">
-        <v>229</v>
-      </c>
-      <c r="B13" s="21" t="s">
-        <v>192</v>
-      </c>
-      <c r="C13" s="22" t="s">
-        <v>148</v>
-      </c>
-      <c r="D13" s="23" t="s">
-        <v>230</v>
-      </c>
-      <c r="E13" s="23" t="s">
-        <v>231</v>
-      </c>
-      <c r="F13" s="23" t="s">
-        <v>232</v>
-      </c>
-      <c r="G13" s="23"/>
-      <c r="H13" s="23" t="s">
-        <v>148</v>
-      </c>
-    </row>
-    <row r="14" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="21" t="s">
-        <v>48</v>
-      </c>
-      <c r="B14" s="21" t="s">
-        <v>193</v>
-      </c>
-      <c r="C14" s="22" t="s">
-        <v>233</v>
-      </c>
-      <c r="D14" s="23" t="s">
-        <v>234</v>
-      </c>
-      <c r="E14" s="23" t="s">
-        <v>235</v>
-      </c>
-      <c r="F14" s="23" t="s">
-        <v>236</v>
-      </c>
-      <c r="G14" s="23" t="s">
-        <v>237</v>
-      </c>
-      <c r="H14" s="23" t="s">
-        <v>155</v>
-      </c>
-    </row>
-    <row r="15" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="21" t="s">
-        <v>238</v>
-      </c>
-      <c r="B15" s="21" t="s">
-        <v>199</v>
-      </c>
-      <c r="C15" s="22" t="s">
-        <v>155</v>
-      </c>
-      <c r="D15" s="23" t="s">
-        <v>239</v>
-      </c>
-      <c r="E15" s="23" t="s">
-        <v>240</v>
-      </c>
-      <c r="F15" s="23" t="s">
-        <v>241</v>
-      </c>
-      <c r="G15" s="23" t="s">
-        <v>242</v>
-      </c>
-      <c r="H15" s="23" t="s">
-        <v>155</v>
-      </c>
-    </row>
-    <row r="16" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="21" t="s">
-        <v>243</v>
-      </c>
-      <c r="B16" s="21" t="s">
-        <v>206</v>
-      </c>
-      <c r="C16" s="22" t="s">
-        <v>244</v>
-      </c>
-      <c r="D16" s="23" t="s">
-        <v>245</v>
-      </c>
-      <c r="E16" s="23" t="s">
-        <v>246</v>
-      </c>
-      <c r="F16" s="23" t="s">
-        <v>247</v>
-      </c>
-      <c r="G16" s="23" t="s">
-        <v>248</v>
-      </c>
-      <c r="H16" s="23" t="s">
-        <v>155</v>
-      </c>
-    </row>
-    <row r="17" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="21" t="s">
-        <v>54</v>
-      </c>
-      <c r="B17" s="21" t="s">
-        <v>213</v>
-      </c>
-      <c r="C17" s="22" t="s">
-        <v>249</v>
-      </c>
-      <c r="D17" s="23" t="s">
-        <v>250</v>
-      </c>
-      <c r="E17" s="23" t="s">
-        <v>251</v>
-      </c>
-      <c r="F17" s="23" t="s">
-        <v>252</v>
-      </c>
-      <c r="G17" s="8" t="s">
-        <v>253</v>
-      </c>
-      <c r="H17" s="23" t="s">
-        <v>254</v>
-      </c>
-    </row>
-    <row r="18" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="21" t="s">
-        <v>255</v>
-      </c>
-      <c r="B18" s="21" t="s">
-        <v>218</v>
-      </c>
-      <c r="C18" s="22" t="s">
-        <v>256</v>
-      </c>
-      <c r="D18" s="23" t="s">
-        <v>257</v>
-      </c>
-      <c r="E18" s="23" t="s">
-        <v>258</v>
-      </c>
-      <c r="F18" s="23" t="s">
-        <v>259</v>
-      </c>
-      <c r="G18" s="23" t="s">
-        <v>260</v>
-      </c>
-      <c r="H18" s="23" t="s">
-        <v>254</v>
-      </c>
-    </row>
-    <row r="19" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="21" t="s">
-        <v>261</v>
-      </c>
-      <c r="B19" s="21" t="s">
-        <v>186</v>
-      </c>
-      <c r="C19" s="22" t="s">
-        <v>254</v>
-      </c>
-      <c r="D19" s="23" t="s">
-        <v>262</v>
-      </c>
-      <c r="E19" s="23" t="s">
-        <v>263</v>
-      </c>
-      <c r="F19" s="23" t="s">
-        <v>264</v>
-      </c>
-      <c r="G19" s="23" t="s">
-        <v>265</v>
-      </c>
-      <c r="H19" s="23" t="s">
-        <v>254</v>
-      </c>
-    </row>
-    <row r="20" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="21" t="s">
-        <v>62</v>
-      </c>
-      <c r="B20" s="21" t="s">
-        <v>192</v>
-      </c>
-      <c r="C20" s="22" t="s">
-        <v>266</v>
-      </c>
-      <c r="D20" s="23" t="s">
-        <v>267</v>
-      </c>
-      <c r="E20" s="23" t="s">
-        <v>268</v>
-      </c>
-      <c r="F20" s="23" t="s">
-        <v>269</v>
-      </c>
-      <c r="G20" s="23" t="s">
-        <v>270</v>
-      </c>
-      <c r="H20" s="23" t="s">
-        <v>271</v>
-      </c>
-    </row>
-    <row r="21" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="21" t="s">
-        <v>70</v>
-      </c>
-      <c r="B21" s="21" t="s">
-        <v>193</v>
-      </c>
-      <c r="C21" s="22" t="s">
-        <v>272</v>
-      </c>
-      <c r="D21" s="23" t="s">
-        <v>273</v>
-      </c>
-      <c r="E21" s="23" t="s">
-        <v>274</v>
-      </c>
-      <c r="F21" s="23" t="s">
-        <v>275</v>
-      </c>
-      <c r="G21" s="23" t="s">
-        <v>276</v>
-      </c>
-      <c r="H21" s="23" t="s">
-        <v>168</v>
-      </c>
-    </row>
-    <row r="22" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="21" t="s">
-        <v>85</v>
-      </c>
-      <c r="B22" s="21" t="s">
-        <v>199</v>
-      </c>
-      <c r="C22" s="22" t="s">
-        <v>168</v>
-      </c>
-      <c r="D22" s="23" t="s">
-        <v>277</v>
-      </c>
-      <c r="E22" s="23" t="s">
-        <v>278</v>
-      </c>
-      <c r="F22" s="23" t="s">
-        <v>279</v>
-      </c>
-      <c r="G22" s="23" t="s">
-        <v>280</v>
-      </c>
-      <c r="H22" s="23" t="s">
-        <v>168</v>
-      </c>
-    </row>
-    <row r="23" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="18" t="s">
-        <v>91</v>
-      </c>
-      <c r="B23" s="18" t="s">
-        <v>206</v>
-      </c>
-      <c r="C23" s="19" t="s">
-        <v>281</v>
-      </c>
-      <c r="D23" s="20" t="s">
-        <v>282</v>
-      </c>
-      <c r="E23" s="20" t="s">
-        <v>283</v>
-      </c>
-      <c r="F23" s="20" t="s">
-        <v>284</v>
-      </c>
-      <c r="G23" s="20" t="s">
-        <v>285</v>
-      </c>
-      <c r="H23" s="20" t="s">
-        <v>198</v>
-      </c>
-    </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="18" t="s">
-        <v>98</v>
-      </c>
-      <c r="B24" s="18" t="s">
-        <v>213</v>
-      </c>
-      <c r="C24" s="19" t="s">
-        <v>286</v>
-      </c>
-      <c r="D24" s="20" t="s">
-        <v>201</v>
-      </c>
-      <c r="E24" s="20" t="s">
-        <v>287</v>
-      </c>
-      <c r="F24" s="20" t="s">
-        <v>288</v>
-      </c>
-      <c r="G24" s="20" t="s">
-        <v>289</v>
-      </c>
-      <c r="H24" s="20" t="s">
-        <v>172</v>
-      </c>
-    </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="18" t="s">
-        <v>99</v>
-      </c>
-      <c r="B25" s="18" t="s">
-        <v>218</v>
-      </c>
-      <c r="C25" s="19" t="s">
-        <v>290</v>
-      </c>
-      <c r="D25" s="20" t="s">
+      <c r="C25" s="16" t="s">
         <v>291</v>
       </c>
-      <c r="E25" s="20" t="s">
-        <v>60</v>
-      </c>
-      <c r="F25" s="20" t="s">
-        <v>60</v>
-      </c>
-      <c r="G25" s="20" t="s">
+      <c r="D25" s="17" t="s">
         <v>292</v>
       </c>
-      <c r="H25" s="20" t="s">
+      <c r="E25" s="17" t="s">
+        <v>188</v>
+      </c>
+      <c r="F25" s="17" t="s">
+        <v>188</v>
+      </c>
+      <c r="G25" s="17" t="s">
         <v>293</v>
+      </c>
+      <c r="H25" s="17" t="s">
+        <v>294</v>
       </c>
     </row>
   </sheetData>
@@ -3303,7 +3294,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F33"/>
+  <dimension ref="A1:F34"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="16"/>
@@ -3316,26 +3307,26 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="E4" s="3" t="s">
         <v>10</v>
@@ -3349,42 +3340,42 @@
         <v>1</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>60</v>
-      </c>
-      <c r="D5" s="24" t="s">
-        <v>301</v>
+        <v>188</v>
+      </c>
+      <c r="D5" s="21" t="s">
+        <v>302</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="F5" s="5" t="s">
-        <v>303</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>304</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="n">
         <v>2</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>305</v>
-      </c>
-      <c r="D6" s="24" t="s">
-        <v>301</v>
+        <v>188</v>
+      </c>
+      <c r="D6" s="21" t="s">
+        <v>302</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>158</v>
+        <v>303</v>
       </c>
       <c r="F6" s="5" t="s">
         <v>306</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="4" t="n">
         <v>3</v>
       </c>
@@ -3392,36 +3383,36 @@
         <v>307</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>60</v>
-      </c>
-      <c r="D7" s="24" t="s">
-        <v>301</v>
+        <v>308</v>
+      </c>
+      <c r="D7" s="21" t="s">
+        <v>302</v>
       </c>
       <c r="E7" s="4" t="s">
-        <v>302</v>
+        <v>158</v>
       </c>
       <c r="F7" s="5" t="s">
-        <v>308</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>309</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="n">
         <v>4</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>60</v>
-      </c>
-      <c r="D8" s="24" t="s">
-        <v>301</v>
+        <v>188</v>
+      </c>
+      <c r="D8" s="21" t="s">
+        <v>302</v>
       </c>
       <c r="E8" s="4" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="F8" s="5" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3429,16 +3420,16 @@
         <v>5</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>312</v>
-      </c>
-      <c r="D9" s="24" t="s">
-        <v>301</v>
+        <v>188</v>
+      </c>
+      <c r="D9" s="21" t="s">
+        <v>302</v>
       </c>
       <c r="E9" s="4" t="s">
-        <v>158</v>
+        <v>303</v>
       </c>
       <c r="F9" s="5" t="s">
         <v>313</v>
@@ -3452,16 +3443,16 @@
         <v>314</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>60</v>
-      </c>
-      <c r="D10" s="24" t="s">
-        <v>301</v>
+        <v>315</v>
+      </c>
+      <c r="D10" s="21" t="s">
+        <v>302</v>
       </c>
       <c r="E10" s="4" t="s">
-        <v>302</v>
+        <v>158</v>
       </c>
       <c r="F10" s="5" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3469,22 +3460,22 @@
         <v>7</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>317</v>
-      </c>
-      <c r="D11" s="24" t="s">
-        <v>301</v>
+        <v>188</v>
+      </c>
+      <c r="D11" s="21" t="s">
+        <v>302</v>
       </c>
       <c r="E11" s="4" t="s">
-        <v>158</v>
+        <v>303</v>
       </c>
       <c r="F11" s="5" t="s">
         <v>318</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="4" t="n">
         <v>8</v>
       </c>
@@ -3494,8 +3485,8 @@
       <c r="C12" s="4" t="s">
         <v>320</v>
       </c>
-      <c r="D12" s="24" t="s">
-        <v>301</v>
+      <c r="D12" s="21" t="s">
+        <v>302</v>
       </c>
       <c r="E12" s="4" t="s">
         <v>158</v>
@@ -3504,7 +3495,7 @@
         <v>321</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="13" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="4" t="n">
         <v>9</v>
       </c>
@@ -3514,14 +3505,14 @@
       <c r="C13" s="4" t="s">
         <v>323</v>
       </c>
-      <c r="D13" s="4" t="s">
-        <v>324</v>
+      <c r="D13" s="21" t="s">
+        <v>302</v>
       </c>
       <c r="E13" s="4" t="s">
         <v>158</v>
       </c>
       <c r="F13" s="5" t="s">
-        <v>318</v>
+        <v>324</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3535,13 +3526,13 @@
         <v>326</v>
       </c>
       <c r="D14" s="4" t="s">
-        <v>324</v>
+        <v>327</v>
       </c>
       <c r="E14" s="4" t="s">
         <v>158</v>
       </c>
       <c r="F14" s="5" t="s">
-        <v>327</v>
+        <v>321</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3554,8 +3545,8 @@
       <c r="C15" s="4" t="s">
         <v>329</v>
       </c>
-      <c r="D15" s="24" t="s">
-        <v>301</v>
+      <c r="D15" s="4" t="s">
+        <v>327</v>
       </c>
       <c r="E15" s="4" t="s">
         <v>158</v>
@@ -3574,8 +3565,8 @@
       <c r="C16" s="4" t="s">
         <v>332</v>
       </c>
-      <c r="D16" s="4" t="s">
-        <v>324</v>
+      <c r="D16" s="21" t="s">
+        <v>302</v>
       </c>
       <c r="E16" s="4" t="s">
         <v>158</v>
@@ -3592,10 +3583,10 @@
         <v>334</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>317</v>
+        <v>335</v>
       </c>
       <c r="D17" s="4" t="s">
-        <v>335</v>
+        <v>327</v>
       </c>
       <c r="E17" s="4" t="s">
         <v>158</v>
@@ -3612,10 +3603,10 @@
         <v>337</v>
       </c>
       <c r="C18" s="4" t="s">
+        <v>320</v>
+      </c>
+      <c r="D18" s="4" t="s">
         <v>338</v>
-      </c>
-      <c r="D18" s="4" t="s">
-        <v>335</v>
       </c>
       <c r="E18" s="4" t="s">
         <v>158</v>
@@ -3632,16 +3623,16 @@
         <v>340</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>320</v>
+        <v>341</v>
       </c>
       <c r="D19" s="4" t="s">
-        <v>324</v>
+        <v>338</v>
       </c>
       <c r="E19" s="4" t="s">
         <v>158</v>
       </c>
       <c r="F19" s="5" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3649,33 +3640,33 @@
         <v>16</v>
       </c>
       <c r="B20" s="5" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="C20" s="4" t="s">
         <v>323</v>
       </c>
       <c r="D20" s="4" t="s">
-        <v>324</v>
+        <v>327</v>
       </c>
       <c r="E20" s="4" t="s">
         <v>158</v>
       </c>
       <c r="F20" s="5" t="s">
-        <v>343</v>
-      </c>
-    </row>
-    <row r="21" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>344</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="4" t="n">
         <v>17</v>
       </c>
       <c r="B21" s="5" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>345</v>
+        <v>326</v>
       </c>
       <c r="D21" s="4" t="s">
-        <v>324</v>
+        <v>327</v>
       </c>
       <c r="E21" s="4" t="s">
         <v>158</v>
@@ -3684,7 +3675,7 @@
         <v>346</v>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="22" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="4" t="n">
         <v>18</v>
       </c>
@@ -3692,16 +3683,16 @@
         <v>347</v>
       </c>
       <c r="C22" s="4" t="s">
-        <v>345</v>
+        <v>348</v>
       </c>
       <c r="D22" s="4" t="s">
-        <v>324</v>
+        <v>327</v>
       </c>
       <c r="E22" s="4" t="s">
         <v>158</v>
       </c>
       <c r="F22" s="5" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3709,19 +3700,19 @@
         <v>19</v>
       </c>
       <c r="B23" s="5" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="C23" s="4" t="s">
-        <v>323</v>
-      </c>
-      <c r="D23" s="24" t="s">
-        <v>301</v>
+        <v>348</v>
+      </c>
+      <c r="D23" s="4" t="s">
+        <v>327</v>
       </c>
       <c r="E23" s="4" t="s">
         <v>158</v>
       </c>
       <c r="F23" s="5" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3729,19 +3720,19 @@
         <v>20</v>
       </c>
       <c r="B24" s="5" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="C24" s="4" t="s">
-        <v>323</v>
-      </c>
-      <c r="D24" s="4" t="s">
-        <v>324</v>
+        <v>326</v>
+      </c>
+      <c r="D24" s="21" t="s">
+        <v>302</v>
       </c>
       <c r="E24" s="4" t="s">
         <v>158</v>
       </c>
       <c r="F24" s="5" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3749,19 +3740,19 @@
         <v>21</v>
       </c>
       <c r="B25" s="5" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="C25" s="4" t="s">
         <v>326</v>
       </c>
       <c r="D25" s="4" t="s">
-        <v>324</v>
+        <v>327</v>
       </c>
       <c r="E25" s="4" t="s">
         <v>158</v>
       </c>
       <c r="F25" s="5" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3769,39 +3760,39 @@
         <v>22</v>
       </c>
       <c r="B26" s="5" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="C26" s="4" t="s">
-        <v>60</v>
+        <v>329</v>
       </c>
       <c r="D26" s="4" t="s">
-        <v>335</v>
+        <v>327</v>
       </c>
       <c r="E26" s="4" t="s">
-        <v>302</v>
+        <v>158</v>
       </c>
       <c r="F26" s="5" t="s">
-        <v>356</v>
-      </c>
-    </row>
-    <row r="27" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="4" t="n">
         <v>23</v>
       </c>
       <c r="B27" s="5" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="C27" s="4" t="s">
-        <v>320</v>
+        <v>188</v>
       </c>
       <c r="D27" s="4" t="s">
-        <v>324</v>
+        <v>338</v>
       </c>
       <c r="E27" s="4" t="s">
-        <v>158</v>
+        <v>303</v>
       </c>
       <c r="F27" s="5" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3809,59 +3800,79 @@
         <v>24</v>
       </c>
       <c r="B28" s="5" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="C28" s="4" t="s">
-        <v>312</v>
+        <v>323</v>
       </c>
       <c r="D28" s="4" t="s">
-        <v>335</v>
+        <v>327</v>
       </c>
       <c r="E28" s="4" t="s">
         <v>158</v>
       </c>
       <c r="F28" s="5" t="s">
-        <v>360</v>
-      </c>
-    </row>
-    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="15" t="s">
         <v>361</v>
       </c>
-      <c r="B30" s="25" t="n">
-        <f aca="false">COUNTIF(E5:E28,"Concluído")</f>
-        <v>5</v>
+    </row>
+    <row r="29" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="4" t="n">
+        <v>25</v>
+      </c>
+      <c r="B29" s="5" t="s">
+        <v>362</v>
+      </c>
+      <c r="C29" s="4" t="s">
+        <v>315</v>
+      </c>
+      <c r="D29" s="4" t="s">
+        <v>338</v>
+      </c>
+      <c r="E29" s="4" t="s">
+        <v>158</v>
+      </c>
+      <c r="F29" s="5" t="s">
+        <v>363</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="15" t="s">
-        <v>362</v>
-      </c>
-      <c r="B31" s="25" t="n">
-        <f aca="false">COUNTIF(E5:E28,"Em andamento")</f>
+      <c r="A31" s="12" t="s">
+        <v>364</v>
+      </c>
+      <c r="B31" s="22" t="n">
+        <f aca="false">COUNTIF(E5:E29,"Concluído")</f>
+        <v>6</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="12" t="s">
+        <v>365</v>
+      </c>
+      <c r="B32" s="22" t="n">
+        <f aca="false">COUNTIF(E5:E29,"Em andamento")</f>
         <v>0</v>
       </c>
     </row>
-    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="15" t="s">
-        <v>363</v>
-      </c>
-      <c r="B32" s="25" t="n">
-        <f aca="false">COUNTIF(E5:E28,"Pendente")</f>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="12" t="s">
+        <v>366</v>
+      </c>
+      <c r="B33" s="22" t="n">
+        <f aca="false">COUNTIF(E5:E29,"Pendente")</f>
         <v>19</v>
       </c>
     </row>
-    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="15" t="s">
-        <v>364</v>
-      </c>
-      <c r="B33" s="26" t="n">
-        <f aca="false">IFERROR(B30/COUNTA(B5:B28),0)</f>
-        <v>0.208333333333333</v>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="12" t="s">
+        <v>367</v>
+      </c>
+      <c r="B34" s="23" t="n">
+        <f aca="false">IFERROR(B31/COUNTA(B5:B29),0)</f>
+        <v>0.24</v>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="A5:F28">
+  <conditionalFormatting sqref="A5:F29">
     <cfRule type="expression" priority="2" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
       <formula>$E5="Concluído"</formula>
     </cfRule>
@@ -3870,7 +3881,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="E5:E28" type="list">
+    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="E5:E29" type="list">
       <formula1>"Pendente,Em andamento,Concluído"</formula1>
       <formula2>0</formula2>
     </dataValidation>

</xml_diff>

<commit_message>
Add Baku hostel (Sahil Bay) and detailed Azerbaijan days
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FbPxpFjYDQnzNa7KTrLMWP
</commit_message>
<xml_diff>
--- a/Eurasia/Roteiro_Eurasia.xlsx
+++ b/Eurasia/Roteiro_Eurasia.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="554" uniqueCount="368">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="555" uniqueCount="370">
   <si>
     <t xml:space="preserve">Itinerário de Voos</t>
   </si>
@@ -493,27 +493,30 @@
     <t xml:space="preserve">Baku</t>
   </si>
   <si>
-    <t xml:space="preserve">Chega ~16:30 (25/10) / sai ~18:00 (28/10)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cidade Velha (Icherisheher) ou Nizami</t>
+    <t xml:space="preserve">Chega ~17:00 (25/10) / sai ~18:00 (28/10)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sahil / Bulvar</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sahil Bay Hostel</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sahil Bay Hostel, Zarifa Aliyeva 27 (antigo Sahil Hostel &amp; Hotel). 600 m da Praça do Chafariz. Pedir para guardar as mochilas no dia 28.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tbilisi (grupo, 4 pessoas)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chega ~22:30 (28/10) / meninos saem ~03:30 (31/10)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cidade Velha ou Sololaki</t>
   </si>
   <si>
     <t xml:space="preserve">Pendente</t>
   </si>
   <si>
-    <t xml:space="preserve">Pedir para guardar as mochilas no dia 28 até a saída para o aeroporto.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tbilisi (grupo, 4 pessoas)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Chega ~22:30 (28/10) / meninos saem ~03:30 (31/10)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cidade Velha ou Sololaki</t>
-  </si>
-  <si>
     <t xml:space="preserve">Confirmar check-in tardio e saída de madrugada dos meninos (voo 06:00).</t>
   </si>
   <si>
@@ -730,28 +733,28 @@
     <t xml:space="preserve">Budapeste → Baku</t>
   </si>
   <si>
-    <t xml:space="preserve">Café da manhã; sair ~09:45 para o aeroporto.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Voo; chegada 15:50.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bulvar, Cidade Velha (Icherisheher) e Flame Towers iluminadas.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">W6 2365 BUD 12:15 → GYD 15:50. E-visa ASAN em mãos.</t>
+    <t xml:space="preserve">Café da manhã; sair ~09:30 para o aeroporto (100E na Deák tér).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Voo; chegada 15:50. No aeroporto: BakuCard e manat; Bolt até o Sahil Bay.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bulvar, Praça do Chafariz, Cidade Velha iluminada e Flame Towers.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">W6 2365 BUD 12:15 → GYD 15:50. E-visa ASAN em mãos. Fim do horário de verão europeu nesta madrugada.</t>
   </si>
   <si>
     <t xml:space="preserve">26/10/2026</t>
   </si>
   <si>
-    <t xml:space="preserve">Cidade Velha: Torre da Donzela, Palácio dos Shirvanshahs.</t>
+    <t xml:space="preserve">Cidade Velha: Torre da Donzela, Palácio dos Shirvanshahs, caravançarás. Almoço: plov, qutab, dolma.</t>
   </si>
   <si>
     <t xml:space="preserve">Museu do Tapete; funicular até o Parque Highland.</t>
   </si>
   <si>
-    <t xml:space="preserve">Jantar azerbaijano na Cidade Velha.</t>
+    <t xml:space="preserve">Yanar Dag depois de escurecer (~30 min de Bolt).</t>
   </si>
   <si>
     <t xml:space="preserve">Centro Heydar Aliyev costuma fechar às segundas.</t>
@@ -763,16 +766,16 @@
     <t xml:space="preserve">Baku (arredores)</t>
   </si>
   <si>
-    <t xml:space="preserve">Gobustan (petróglifos, UNESCO) + vulcões de lama.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ateshgah (templo do fogo).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Yanar Dag ao pôr do sol.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tour ou motorista privado (dia inteiro).</t>
+    <t xml:space="preserve">Gobustan (petróglifos, UNESCO) + vulcões de lama (Lada local a partir da vila).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ateshgah (templo do fogo, Surakhani).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jantar no centro.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tour em grupo ou motorista privado (dia inteiro). Levar manat em dinheiro.</t>
   </si>
   <si>
     <t xml:space="preserve">Baku → Tbilisi</t>
@@ -985,58 +988,61 @@
     <t xml:space="preserve">Reservar hostel Baku (25 a 28/10)</t>
   </si>
   <si>
+    <t xml:space="preserve">Sahil Bay Hostel. Preencher localizador e valor na aba Hospedagem.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Reservar hostel Tbilisi (grupo 28 a 31/10 + Diego 31/10 a 01/11)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Até 25/10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Check-in ~22:30 no dia 28. Ver aba Hospedagem.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Reservar hostel Atenas (31/10 a 03/11)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Até 28/10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Média</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ver aba Hospedagem.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Reservar pernoite São Paulo (04 a 05/11)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Até 01/11</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Se não houver onde ficar. Ver aba Hospedagem.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ingresso Jardim Majorelle (21/10)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hoje</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Só online, com horário marcado.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Visita guiada Parlamento de Budapeste (23/10)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">21/10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Esgota com antecedência; escolher horário em inglês ou espanhol.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ingresso Termas Széchenyi (23/10)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Até 23/10</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ver aba Hospedagem.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Reservar hostel Tbilisi (grupo 28 a 31/10 + Diego 31/10 a 01/11)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Até 25/10</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Check-in ~22:30 no dia 28. Ver aba Hospedagem.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Reservar hostel Atenas (31/10 a 03/11)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Até 28/10</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Média</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Reservar pernoite São Paulo (04 a 05/11)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Até 01/11</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Se não houver onde ficar. Ver aba Hospedagem.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ingresso Jardim Majorelle (21/10)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Hoje</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Só online, com horário marcado.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Visita guiada Parlamento de Budapeste (23/10)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">21/10</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Esgota com antecedência; escolher horário em inglês ou espanhol.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ingresso Termas Széchenyi (23/10)</t>
   </si>
   <si>
     <t xml:space="preserve">Baixa</t>
@@ -2488,7 +2494,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="8" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="7" t="s">
         <v>155</v>
       </c>
@@ -2508,11 +2514,13 @@
       <c r="F8" s="5" t="s">
         <v>157</v>
       </c>
-      <c r="G8" s="6"/>
+      <c r="G8" s="6" t="s">
+        <v>158</v>
+      </c>
       <c r="H8" s="6"/>
       <c r="I8" s="11"/>
       <c r="J8" s="4" t="s">
-        <v>158</v>
+        <v>144</v>
       </c>
       <c r="K8" s="5" t="s">
         <v>159</v>
@@ -2542,15 +2550,15 @@
       <c r="H9" s="6"/>
       <c r="I9" s="11"/>
       <c r="J9" s="4" t="s">
-        <v>158</v>
+        <v>163</v>
       </c>
       <c r="K9" s="5" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="7" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="B10" s="8" t="n">
         <v>46326</v>
@@ -2563,24 +2571,24 @@
         <v>1</v>
       </c>
       <c r="E10" s="5" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="F10" s="5" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="G10" s="6"/>
       <c r="H10" s="6"/>
       <c r="I10" s="11"/>
       <c r="J10" s="4" t="s">
-        <v>158</v>
+        <v>163</v>
       </c>
       <c r="K10" s="5" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="7" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="B11" s="8" t="n">
         <v>46326</v>
@@ -2593,24 +2601,24 @@
         <v>3</v>
       </c>
       <c r="E11" s="5" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="F11" s="5" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="G11" s="6"/>
       <c r="H11" s="6"/>
       <c r="I11" s="11"/>
       <c r="J11" s="4" t="s">
-        <v>158</v>
+        <v>163</v>
       </c>
       <c r="K11" s="5" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="7" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="B12" s="8" t="n">
         <v>46330</v>
@@ -2623,24 +2631,24 @@
         <v>1</v>
       </c>
       <c r="E12" s="5" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="F12" s="5" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="G12" s="6"/>
       <c r="H12" s="6"/>
       <c r="I12" s="11"/>
       <c r="J12" s="4" t="s">
-        <v>158</v>
+        <v>163</v>
       </c>
       <c r="K12" s="5" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="12" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="B13" s="13"/>
       <c r="C13" s="13"/>
@@ -2655,7 +2663,7 @@
       <c r="I13" s="13"/>
       <c r="J13" s="13"/>
       <c r="K13" s="14" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
     </row>
   </sheetData>
@@ -2702,12 +2710,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2715,25 +2723,25 @@
         <v>2</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="C4" s="3" t="s">
         <v>130</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2741,49 +2749,49 @@
         <v>12</v>
       </c>
       <c r="B5" s="15" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="C5" s="16" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="D5" s="17" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="E5" s="17" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="F5" s="17" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="G5" s="17" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="H5" s="17" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="15" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="B6" s="15" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="C6" s="16" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="D6" s="17" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="E6" s="17" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="F6" s="17" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="G6" s="17"/>
       <c r="H6" s="17" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2791,25 +2799,25 @@
         <v>20</v>
       </c>
       <c r="B7" s="15" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="C7" s="16" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="D7" s="17" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="E7" s="17" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="F7" s="17" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="G7" s="17" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="H7" s="17" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2817,25 +2825,25 @@
         <v>29</v>
       </c>
       <c r="B8" s="15" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="C8" s="16" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="D8" s="17" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="E8" s="17" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="F8" s="17" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="G8" s="17" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="H8" s="17" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2843,22 +2851,22 @@
         <v>34</v>
       </c>
       <c r="B9" s="18" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="C9" s="19" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="D9" s="20" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="E9" s="20" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="F9" s="20" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="G9" s="20" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="H9" s="20" t="s">
         <v>139</v>
@@ -2866,25 +2874,25 @@
     </row>
     <row r="10" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="18" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="B10" s="18" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="C10" s="19" t="s">
         <v>139</v>
       </c>
       <c r="D10" s="20" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="E10" s="20" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="F10" s="20" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="G10" s="20" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="H10" s="20" t="s">
         <v>139</v>
@@ -2895,22 +2903,22 @@
         <v>41</v>
       </c>
       <c r="B11" s="18" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="C11" s="19" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="D11" s="20" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="E11" s="20" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="F11" s="20" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="G11" s="20" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="H11" s="20" t="s">
         <v>148</v>
@@ -2918,25 +2926,25 @@
     </row>
     <row r="12" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="18" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="B12" s="18" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="C12" s="19" t="s">
         <v>148</v>
       </c>
       <c r="D12" s="20" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="E12" s="20" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="F12" s="20" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="G12" s="20" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="H12" s="20" t="s">
         <v>148</v>
@@ -2944,75 +2952,75 @@
     </row>
     <row r="13" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="18" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="B13" s="18" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="C13" s="19" t="s">
         <v>148</v>
       </c>
       <c r="D13" s="20" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="E13" s="20" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="F13" s="20" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="G13" s="20"/>
       <c r="H13" s="20" t="s">
         <v>148</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="14" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="18" t="s">
         <v>48</v>
       </c>
       <c r="B14" s="18" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="C14" s="19" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="D14" s="20" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="E14" s="20" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="F14" s="20" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="G14" s="20" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="H14" s="20" t="s">
         <v>155</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="15" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="18" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="B15" s="18" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="C15" s="19" t="s">
         <v>155</v>
       </c>
       <c r="D15" s="20" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="E15" s="20" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="F15" s="20" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="G15" s="20" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="H15" s="20" t="s">
         <v>155</v>
@@ -3020,25 +3028,25 @@
     </row>
     <row r="16" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="18" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="B16" s="18" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="C16" s="19" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="D16" s="20" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="E16" s="20" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="F16" s="20" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="G16" s="20" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="H16" s="20" t="s">
         <v>155</v>
@@ -3049,77 +3057,77 @@
         <v>54</v>
       </c>
       <c r="B17" s="18" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="C17" s="19" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="D17" s="20" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="E17" s="20" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="F17" s="20" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="G17" s="20" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="H17" s="20" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="18" t="s">
+        <v>257</v>
+      </c>
+      <c r="B18" s="18" t="s">
+        <v>220</v>
+      </c>
+      <c r="C18" s="19" t="s">
+        <v>258</v>
+      </c>
+      <c r="D18" s="20" t="s">
+        <v>259</v>
+      </c>
+      <c r="E18" s="20" t="s">
+        <v>260</v>
+      </c>
+      <c r="F18" s="20" t="s">
+        <v>261</v>
+      </c>
+      <c r="G18" s="20" t="s">
+        <v>262</v>
+      </c>
+      <c r="H18" s="20" t="s">
         <v>256</v>
-      </c>
-      <c r="B18" s="18" t="s">
-        <v>219</v>
-      </c>
-      <c r="C18" s="19" t="s">
-        <v>257</v>
-      </c>
-      <c r="D18" s="20" t="s">
-        <v>258</v>
-      </c>
-      <c r="E18" s="20" t="s">
-        <v>259</v>
-      </c>
-      <c r="F18" s="20" t="s">
-        <v>260</v>
-      </c>
-      <c r="G18" s="20" t="s">
-        <v>261</v>
-      </c>
-      <c r="H18" s="20" t="s">
-        <v>255</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="18" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="B19" s="18" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="C19" s="19" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="D19" s="20" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="E19" s="20" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="F19" s="20" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="G19" s="20" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="H19" s="20" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3127,25 +3135,25 @@
         <v>61</v>
       </c>
       <c r="B20" s="18" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="C20" s="19" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="D20" s="20" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="E20" s="20" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="F20" s="20" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="G20" s="20" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="H20" s="20" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3153,25 +3161,25 @@
         <v>69</v>
       </c>
       <c r="B21" s="18" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="C21" s="19" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="D21" s="20" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="E21" s="20" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="F21" s="20" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="G21" s="20" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="H21" s="20" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3179,25 +3187,25 @@
         <v>85</v>
       </c>
       <c r="B22" s="18" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="C22" s="19" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="D22" s="20" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="E22" s="20" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="F22" s="20" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="G22" s="20" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="H22" s="20" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3205,25 +3213,25 @@
         <v>91</v>
       </c>
       <c r="B23" s="15" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="C23" s="16" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="D23" s="17" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="E23" s="17" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="F23" s="17" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="G23" s="17" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="H23" s="17" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3231,25 +3239,25 @@
         <v>98</v>
       </c>
       <c r="B24" s="15" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="C24" s="16" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="D24" s="17" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="E24" s="17" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="F24" s="17" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="G24" s="17" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="H24" s="17" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3257,25 +3265,25 @@
         <v>99</v>
       </c>
       <c r="B25" s="15" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="C25" s="16" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="D25" s="17" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="E25" s="17" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="F25" s="17" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="G25" s="17" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="H25" s="17" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
     </row>
   </sheetData>
@@ -3307,26 +3315,26 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="E4" s="3" t="s">
         <v>10</v>
@@ -3340,19 +3348,19 @@
         <v>1</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="D5" s="21" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="F5" s="5" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3360,19 +3368,19 @@
         <v>2</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="D6" s="21" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="F6" s="5" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3380,19 +3388,19 @@
         <v>3</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="D7" s="21" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="E7" s="4" t="s">
-        <v>158</v>
+        <v>163</v>
       </c>
       <c r="F7" s="5" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3400,19 +3408,19 @@
         <v>4</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="D8" s="21" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="E8" s="4" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="F8" s="5" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3420,19 +3428,19 @@
         <v>5</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="D9" s="21" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="E9" s="4" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="F9" s="5" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3440,19 +3448,19 @@
         <v>6</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="D10" s="21" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="E10" s="4" t="s">
-        <v>158</v>
+        <v>163</v>
       </c>
       <c r="F10" s="5" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3460,19 +3468,19 @@
         <v>7</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="D11" s="21" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="E11" s="4" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="F11" s="5" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3480,16 +3488,16 @@
         <v>8</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>320</v>
+        <v>189</v>
       </c>
       <c r="D12" s="21" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="E12" s="4" t="s">
-        <v>158</v>
+        <v>304</v>
       </c>
       <c r="F12" s="5" t="s">
         <v>321</v>
@@ -3506,10 +3514,10 @@
         <v>323</v>
       </c>
       <c r="D13" s="21" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="E13" s="4" t="s">
-        <v>158</v>
+        <v>163</v>
       </c>
       <c r="F13" s="5" t="s">
         <v>324</v>
@@ -3529,10 +3537,10 @@
         <v>327</v>
       </c>
       <c r="E14" s="4" t="s">
-        <v>158</v>
+        <v>163</v>
       </c>
       <c r="F14" s="5" t="s">
-        <v>321</v>
+        <v>328</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3540,19 +3548,19 @@
         <v>11</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="D15" s="4" t="s">
         <v>327</v>
       </c>
       <c r="E15" s="4" t="s">
-        <v>158</v>
+        <v>163</v>
       </c>
       <c r="F15" s="5" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3560,19 +3568,19 @@
         <v>12</v>
       </c>
       <c r="B16" s="5" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="D16" s="21" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="E16" s="4" t="s">
-        <v>158</v>
+        <v>163</v>
       </c>
       <c r="F16" s="5" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3580,19 +3588,19 @@
         <v>13</v>
       </c>
       <c r="B17" s="5" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="D17" s="4" t="s">
         <v>327</v>
       </c>
       <c r="E17" s="4" t="s">
-        <v>158</v>
+        <v>163</v>
       </c>
       <c r="F17" s="5" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3600,19 +3608,19 @@
         <v>14</v>
       </c>
       <c r="B18" s="5" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>320</v>
+        <v>339</v>
       </c>
       <c r="D18" s="4" t="s">
-        <v>338</v>
+        <v>340</v>
       </c>
       <c r="E18" s="4" t="s">
-        <v>158</v>
+        <v>163</v>
       </c>
       <c r="F18" s="5" t="s">
-        <v>339</v>
+        <v>341</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3620,19 +3628,19 @@
         <v>15</v>
       </c>
       <c r="B19" s="5" t="s">
+        <v>342</v>
+      </c>
+      <c r="C19" s="4" t="s">
+        <v>343</v>
+      </c>
+      <c r="D19" s="4" t="s">
         <v>340</v>
       </c>
-      <c r="C19" s="4" t="s">
-        <v>341</v>
-      </c>
-      <c r="D19" s="4" t="s">
-        <v>338</v>
-      </c>
       <c r="E19" s="4" t="s">
-        <v>158</v>
+        <v>163</v>
       </c>
       <c r="F19" s="5" t="s">
-        <v>342</v>
+        <v>344</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3640,7 +3648,7 @@
         <v>16</v>
       </c>
       <c r="B20" s="5" t="s">
-        <v>343</v>
+        <v>345</v>
       </c>
       <c r="C20" s="4" t="s">
         <v>323</v>
@@ -3649,10 +3657,10 @@
         <v>327</v>
       </c>
       <c r="E20" s="4" t="s">
-        <v>158</v>
+        <v>163</v>
       </c>
       <c r="F20" s="5" t="s">
-        <v>344</v>
+        <v>346</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3660,7 +3668,7 @@
         <v>17</v>
       </c>
       <c r="B21" s="5" t="s">
-        <v>345</v>
+        <v>347</v>
       </c>
       <c r="C21" s="4" t="s">
         <v>326</v>
@@ -3669,10 +3677,10 @@
         <v>327</v>
       </c>
       <c r="E21" s="4" t="s">
-        <v>158</v>
+        <v>163</v>
       </c>
       <c r="F21" s="5" t="s">
-        <v>346</v>
+        <v>348</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3680,19 +3688,19 @@
         <v>18</v>
       </c>
       <c r="B22" s="5" t="s">
-        <v>347</v>
+        <v>349</v>
       </c>
       <c r="C22" s="4" t="s">
-        <v>348</v>
+        <v>350</v>
       </c>
       <c r="D22" s="4" t="s">
         <v>327</v>
       </c>
       <c r="E22" s="4" t="s">
-        <v>158</v>
+        <v>163</v>
       </c>
       <c r="F22" s="5" t="s">
-        <v>349</v>
+        <v>351</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3700,19 +3708,19 @@
         <v>19</v>
       </c>
       <c r="B23" s="5" t="s">
+        <v>352</v>
+      </c>
+      <c r="C23" s="4" t="s">
         <v>350</v>
-      </c>
-      <c r="C23" s="4" t="s">
-        <v>348</v>
       </c>
       <c r="D23" s="4" t="s">
         <v>327</v>
       </c>
       <c r="E23" s="4" t="s">
-        <v>158</v>
+        <v>163</v>
       </c>
       <c r="F23" s="5" t="s">
-        <v>351</v>
+        <v>353</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3720,19 +3728,19 @@
         <v>20</v>
       </c>
       <c r="B24" s="5" t="s">
-        <v>352</v>
+        <v>354</v>
       </c>
       <c r="C24" s="4" t="s">
         <v>326</v>
       </c>
       <c r="D24" s="21" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="E24" s="4" t="s">
-        <v>158</v>
+        <v>163</v>
       </c>
       <c r="F24" s="5" t="s">
-        <v>353</v>
+        <v>355</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3740,7 +3748,7 @@
         <v>21</v>
       </c>
       <c r="B25" s="5" t="s">
-        <v>354</v>
+        <v>356</v>
       </c>
       <c r="C25" s="4" t="s">
         <v>326</v>
@@ -3749,10 +3757,10 @@
         <v>327</v>
       </c>
       <c r="E25" s="4" t="s">
-        <v>158</v>
+        <v>163</v>
       </c>
       <c r="F25" s="5" t="s">
-        <v>355</v>
+        <v>357</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3760,19 +3768,19 @@
         <v>22</v>
       </c>
       <c r="B26" s="5" t="s">
-        <v>356</v>
+        <v>358</v>
       </c>
       <c r="C26" s="4" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="D26" s="4" t="s">
         <v>327</v>
       </c>
       <c r="E26" s="4" t="s">
-        <v>158</v>
+        <v>163</v>
       </c>
       <c r="F26" s="5" t="s">
-        <v>357</v>
+        <v>359</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3780,19 +3788,19 @@
         <v>23</v>
       </c>
       <c r="B27" s="5" t="s">
-        <v>358</v>
+        <v>360</v>
       </c>
       <c r="C27" s="4" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="D27" s="4" t="s">
-        <v>338</v>
+        <v>340</v>
       </c>
       <c r="E27" s="4" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="F27" s="5" t="s">
-        <v>359</v>
+        <v>361</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3800,7 +3808,7 @@
         <v>24</v>
       </c>
       <c r="B28" s="5" t="s">
-        <v>360</v>
+        <v>362</v>
       </c>
       <c r="C28" s="4" t="s">
         <v>323</v>
@@ -3809,10 +3817,10 @@
         <v>327</v>
       </c>
       <c r="E28" s="4" t="s">
-        <v>158</v>
+        <v>163</v>
       </c>
       <c r="F28" s="5" t="s">
-        <v>361</v>
+        <v>363</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3820,33 +3828,33 @@
         <v>25</v>
       </c>
       <c r="B29" s="5" t="s">
-        <v>362</v>
+        <v>364</v>
       </c>
       <c r="C29" s="4" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="D29" s="4" t="s">
-        <v>338</v>
+        <v>340</v>
       </c>
       <c r="E29" s="4" t="s">
-        <v>158</v>
+        <v>163</v>
       </c>
       <c r="F29" s="5" t="s">
-        <v>363</v>
+        <v>365</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="12" t="s">
-        <v>364</v>
+        <v>366</v>
       </c>
       <c r="B31" s="22" t="n">
         <f aca="false">COUNTIF(E5:E29,"Concluído")</f>
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="12" t="s">
-        <v>365</v>
+        <v>367</v>
       </c>
       <c r="B32" s="22" t="n">
         <f aca="false">COUNTIF(E5:E29,"Em andamento")</f>
@@ -3855,20 +3863,20 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="12" t="s">
-        <v>366</v>
+        <v>368</v>
       </c>
       <c r="B33" s="22" t="n">
         <f aca="false">COUNTIF(E5:E29,"Pendente")</f>
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="12" t="s">
-        <v>367</v>
+        <v>369</v>
       </c>
       <c r="B34" s="23" t="n">
         <f aca="false">IFERROR(B31/COUNTA(B5:B29),0)</f>
-        <v>0.24</v>
+        <v>0.28</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Move Yanar Dag to Tuesday 27/10
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FbPxpFjYDQnzNa7KTrLMWP
</commit_message>
<xml_diff>
--- a/Eurasia/Roteiro_Eurasia.xlsx
+++ b/Eurasia/Roteiro_Eurasia.xlsx
@@ -754,7 +754,7 @@
     <t xml:space="preserve">Museu do Tapete; funicular até o Parque Highland.</t>
   </si>
   <si>
-    <t xml:space="preserve">Yanar Dag depois de escurecer (~30 min de Bolt).</t>
+    <t xml:space="preserve">Parque Highland ao anoitecer (vista das Flame Towers acesas); jantar na Nizami ou na Cidade Velha.</t>
   </si>
   <si>
     <t xml:space="preserve">Centro Heydar Aliyev costuma fechar às segundas.</t>
@@ -772,10 +772,10 @@
     <t xml:space="preserve">Ateshgah (templo do fogo, Surakhani).</t>
   </si>
   <si>
-    <t xml:space="preserve">Jantar no centro.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tour em grupo ou motorista privado (dia inteiro). Levar manat em dinheiro.</t>
+    <t xml:space="preserve">Yanar Dag depois de escurecer (~30 min do Ateshgah); volta ao centro para jantar.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tour em grupo ou motorista privado (dia inteiro, incluindo Yanar Dag). Levar manat em dinheiro.</t>
   </si>
   <si>
     <t xml:space="preserve">Baku → Tbilisi</t>
@@ -3026,7 +3026,7 @@
         <v>155</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="16" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="18" t="s">
         <v>245</v>
       </c>

</xml_diff>

<commit_message>
Move Baku museums to 28/10
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FbPxpFjYDQnzNa7KTrLMWP
</commit_message>
<xml_diff>
--- a/Eurasia/Roteiro_Eurasia.xlsx
+++ b/Eurasia/Roteiro_Eurasia.xlsx
@@ -748,16 +748,16 @@
     <t xml:space="preserve">26/10/2026</t>
   </si>
   <si>
-    <t xml:space="preserve">Cidade Velha: Torre da Donzela, Palácio dos Shirvanshahs, caravançarás. Almoço: plov, qutab, dolma.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Museu do Tapete; funicular até o Parque Highland.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Parque Highland ao anoitecer (vista das Flame Towers acesas); jantar na Nizami ou na Cidade Velha.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Centro Heydar Aliyev costuma fechar às segundas.</t>
+    <t xml:space="preserve">Passeio a pé pela Cidade Velha (muralhas, vielas, caravançarás, lojas de tapetes), sem entrar em museus.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bulvar à beira do Cáspio; funicular até o Parque Highland (pôr do sol ~17:20, Alameda dos Mártires).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Flame Towers acesas vistas do Parque Highland; jantar na Cidade Velha; Nizami e Praça do Chafariz.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Museus ficam para 28/10.</t>
   </si>
   <si>
     <t xml:space="preserve">27/10/2026</t>
@@ -781,10 +781,10 @@
     <t xml:space="preserve">Baku → Tbilisi</t>
   </si>
   <si>
-    <t xml:space="preserve">Centro Heydar Aliyev.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Almoço de despedida; sair ~18:00 para GYD.</t>
+    <t xml:space="preserve">Museus: Torre da Donzela, Palácio dos Shirvanshahs e Museu do Tapete.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Centro Heydar Aliyev; sair ~18:00 do hostel para GYD.</t>
   </si>
   <si>
     <t xml:space="preserve">Voo para Tbilisi.</t>

</xml_diff>

<commit_message>
Detail Athens days 01-03/11
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FbPxpFjYDQnzNa7KTrLMWP
</commit_message>
<xml_diff>
--- a/Eurasia/Roteiro_Eurasia.xlsx
+++ b/Eurasia/Roteiro_Eurasia.xlsx
@@ -850,34 +850,34 @@
     <t xml:space="preserve">Tbilisi → Atenas</t>
   </si>
   <si>
-    <t xml:space="preserve">Diego chega 04:15 e encontra os meninos no hostel; descanso.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ney e Claudio: voo ATH → LIS (Claudio segue para Luanda às 22:35). Grupo: Plaka e Anafiotika.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Jantar em Monastiraki com vista da Acrópole.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GQ 785 TBS 02:45 → ATH 04:15.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Acrópole (primeiro horário) e Museu da Acrópole.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ágora Antiga e Templo de Hefesto; Monastiraki.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Pôr do sol no Monte Licabeto.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Acrópole: ingresso online com horário. Claudio chega a GRU às 15:05 (DT 747).</t>
+    <t xml:space="preserve">Chegada 04:15; X95 ou táxi até o hostel; dormir. 11:30 Ágora Antiga e Templo de Hefesto (grátis: 1º domingo do mês).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Almoço em Monastiraki/Psyri. 14:30 Acrópole (grátis hoje; fila; última entrada 16:30). Pôr do sol na colina do Areópago.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Plaka e Anafiotika; jantar. Despedida de Ney e Claudio (voam para Lisboa).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GQ 785 TBS 02:45 → ATH 04:15. Metrô do aeroporto ainda não funciona às 04:15.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">09:00 Museu da Acrópole. Templo de Zeus Olímpico e Arco de Adriano.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Estádio Panatenaico; Jardim Nacional; troca da guarda na Praça Syntagma (de hora em hora).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pôr do sol no Monte Licabeto (funicular); jantar em Psyri ou Koukaki. Dormir cedo.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Alternativa de manhã: Museu Arqueológico Nacional (seg 08:30–15:30).</t>
   </si>
   <si>
     <t xml:space="preserve">Atenas → Lisboa → Luanda</t>
   </si>
   <si>
-    <t xml:space="preserve">Sair ~06:30 para o aeroporto.</t>
+    <t xml:space="preserve">Sair ~06:15 do hostel (metrô linha 3 ou X95) para o aeroporto.</t>
   </si>
   <si>
     <t xml:space="preserve">Lisboa: Chiado, Bairro Alto, Elevador de Santa Justa; LX Factory.</t>
@@ -3182,7 +3182,7 @@
         <v>169</v>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="22" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="18" t="s">
         <v>85</v>
       </c>

</xml_diff>